<commit_message>
add 2019 Hucuktlis ATS estimate
</commit_message>
<xml_diff>
--- a/1. data/Barkley-Sk_pre-smolt_abundances.xlsx
+++ b/1. data/Barkley-Sk_pre-smolt_abundances.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\brownn\Documents\WCVI\Barkley-Sk-CSAS\1. data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45793E4F-63E2-43BF-B8B4-A5720D5BF6D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B3A6A23-78BD-405B-B0CD-A17B2BB718DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{93B9BABA-C468-4873-970E-7D7E9A90394F}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{93B9BABA-C468-4873-970E-7D7E9A90394F}"/>
   </bookViews>
   <sheets>
     <sheet name="ATS_estimates" sheetId="2" r:id="rId1"/>
@@ -46,6 +46,7 @@
     <author>Brown, Nicholas</author>
     <author>tc={9450F348-AFEB-4317-AD43-51976EFBA421}</author>
     <author>tc={C335BF2D-8A76-4A85-B639-EC939DD5E53A}</author>
+    <author>tc={3E6EE213-51C5-4BE7-94A1-C3C937E7343E}</author>
     <author>tc={288476D4-5EF1-4853-B334-5E56430540C8}</author>
     <author>tc={FC5C3F1C-3F41-443B-A044-4AEECF017EAF}</author>
     <author>tc={80809EA6-1C75-4782-B75F-9B8D8E1FF3DD}</author>
@@ -128,7 +129,15 @@
     1977-1985 average CV applied to guesstimated mean</t>
       </text>
     </comment>
-    <comment ref="G211" authorId="4" shapeId="0" xr:uid="{288476D4-5EF1-4853-B334-5E56430540C8}">
+    <comment ref="F211" authorId="4" shapeId="0" xr:uid="{3E6EE213-51C5-4BE7-94A1-C3C937E7343E}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Assuming 50/50 Sk/Stickle. Tows caught 3 Sk, 6 Stickle, but notes indicate they likely hit a pocket of stickles at a shallower depth</t>
+      </text>
+    </comment>
+    <comment ref="G212" authorId="5" shapeId="0" xr:uid="{288476D4-5EF1-4853-B334-5E56430540C8}">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -136,7 +145,7 @@
     Converts 95% CI of the total limnetic fish estimate to a coefficient of variation, and then multiplies that by the species specific estimate to yield and SD value. </t>
       </text>
     </comment>
-    <comment ref="I211" authorId="5" shapeId="0" xr:uid="{FC5C3F1C-3F41-443B-A044-4AEECF017EAF}">
+    <comment ref="I212" authorId="6" shapeId="0" xr:uid="{FC5C3F1C-3F41-443B-A044-4AEECF017EAF}">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -144,7 +153,7 @@
     Converts 95% CI of the total limnetic fish estimate to a coefficient of variation, and then multiplies that by the species specific estimate to yield and SD value. </t>
       </text>
     </comment>
-    <comment ref="G212" authorId="6" shapeId="0" xr:uid="{80809EA6-1C75-4782-B75F-9B8D8E1FF3DD}">
+    <comment ref="G213" authorId="7" shapeId="0" xr:uid="{80809EA6-1C75-4782-B75F-9B8D8E1FF3DD}">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -153,7 +162,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="I212" authorId="7" shapeId="0" xr:uid="{4AD49B9C-A1D0-4A25-B5DF-3F2CF529CCE3}">
+    <comment ref="I213" authorId="8" shapeId="0" xr:uid="{4AD49B9C-A1D0-4A25-B5DF-3F2CF529CCE3}">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -162,7 +171,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="G213" authorId="8" shapeId="0" xr:uid="{C9E6BF89-D9D3-4E3C-B697-A5DC0E655E3C}">
+    <comment ref="G214" authorId="9" shapeId="0" xr:uid="{C9E6BF89-D9D3-4E3C-B697-A5DC0E655E3C}">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -171,7 +180,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="I213" authorId="9" shapeId="0" xr:uid="{30CBB802-82F2-45BB-8B27-7315D97962A6}">
+    <comment ref="I214" authorId="10" shapeId="0" xr:uid="{30CBB802-82F2-45BB-8B27-7315D97962A6}">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -180,7 +189,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="G214" authorId="10" shapeId="0" xr:uid="{1FC59F05-C26A-4351-8236-C828500ADDBC}">
+    <comment ref="G215" authorId="11" shapeId="0" xr:uid="{1FC59F05-C26A-4351-8236-C828500ADDBC}">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -189,7 +198,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="I214" authorId="11" shapeId="0" xr:uid="{1348B42C-4137-429B-A693-D62CB5C3BC03}">
+    <comment ref="I215" authorId="12" shapeId="0" xr:uid="{1348B42C-4137-429B-A693-D62CB5C3BC03}">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -198,7 +207,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="J256" authorId="1" shapeId="0" xr:uid="{F52DD24B-5ABC-4F49-A632-F9389FACE903}">
+    <comment ref="J257" authorId="1" shapeId="0" xr:uid="{F52DD24B-5ABC-4F49-A632-F9389FACE903}">
       <text>
         <r>
           <rPr>
@@ -227,7 +236,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="21">
   <si>
     <t>smolt_year</t>
   </si>
@@ -300,7 +309,7 @@
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -342,6 +351,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -409,9 +424,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -449,7 +464,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -555,7 +570,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -697,7 +712,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -714,33 +729,36 @@
   <threadedComment ref="G113" dT="2025-03-04T16:50:12.85" personId="{3DE5C77A-2EC9-410D-AF92-25A6BD2452F6}" id="{C335BF2D-8A76-4A85-B639-EC939DD5E53A}">
     <text>1977-1985 average CV applied to guesstimated mean</text>
   </threadedComment>
-  <threadedComment ref="G211" dT="2025-07-23T21:51:33.73" personId="{3DE5C77A-2EC9-410D-AF92-25A6BD2452F6}" id="{288476D4-5EF1-4853-B334-5E56430540C8}">
+  <threadedComment ref="F211" dT="2026-03-31T23:00:59.33" personId="{3DE5C77A-2EC9-410D-AF92-25A6BD2452F6}" id="{3E6EE213-51C5-4BE7-94A1-C3C937E7343E}">
+    <text>Assuming 50/50 Sk/Stickle. Tows caught 3 Sk, 6 Stickle, but notes indicate they likely hit a pocket of stickles at a shallower depth</text>
+  </threadedComment>
+  <threadedComment ref="G212" dT="2025-07-23T21:51:33.73" personId="{3DE5C77A-2EC9-410D-AF92-25A6BD2452F6}" id="{288476D4-5EF1-4853-B334-5E56430540C8}">
     <text xml:space="preserve">Converts 95% CI of the total limnetic fish estimate to a coefficient of variation, and then multiplies that by the species specific estimate to yield and SD value. </text>
   </threadedComment>
-  <threadedComment ref="I211" dT="2025-07-23T21:51:33.73" personId="{3DE5C77A-2EC9-410D-AF92-25A6BD2452F6}" id="{FC5C3F1C-3F41-443B-A044-4AEECF017EAF}">
+  <threadedComment ref="I212" dT="2025-07-23T21:51:33.73" personId="{3DE5C77A-2EC9-410D-AF92-25A6BD2452F6}" id="{FC5C3F1C-3F41-443B-A044-4AEECF017EAF}">
     <text xml:space="preserve">Converts 95% CI of the total limnetic fish estimate to a coefficient of variation, and then multiplies that by the species specific estimate to yield and SD value. </text>
   </threadedComment>
-  <threadedComment ref="G212" dT="2025-07-23T21:53:41.91" personId="{3DE5C77A-2EC9-410D-AF92-25A6BD2452F6}" id="{80809EA6-1C75-4782-B75F-9B8D8E1FF3DD}">
+  <threadedComment ref="G213" dT="2025-07-23T21:53:41.91" personId="{3DE5C77A-2EC9-410D-AF92-25A6BD2452F6}" id="{80809EA6-1C75-4782-B75F-9B8D8E1FF3DD}">
     <text xml:space="preserve">Converts 95% CI of the total limnetic fish estimate to a coefficient of variation, and then multiplies that by the species specific estimate to yield and SD value. 
 </text>
   </threadedComment>
-  <threadedComment ref="I212" dT="2025-07-23T21:53:41.91" personId="{3DE5C77A-2EC9-410D-AF92-25A6BD2452F6}" id="{4AD49B9C-A1D0-4A25-B5DF-3F2CF529CCE3}">
+  <threadedComment ref="I213" dT="2025-07-23T21:53:41.91" personId="{3DE5C77A-2EC9-410D-AF92-25A6BD2452F6}" id="{4AD49B9C-A1D0-4A25-B5DF-3F2CF529CCE3}">
     <text xml:space="preserve">Converts 95% CI of the total limnetic fish estimate to a coefficient of variation, and then multiplies that by the species specific estimate to yield and SD value. 
 </text>
   </threadedComment>
-  <threadedComment ref="G213" dT="2025-07-23T21:53:45.87" personId="{3DE5C77A-2EC9-410D-AF92-25A6BD2452F6}" id="{C9E6BF89-D9D3-4E3C-B697-A5DC0E655E3C}">
+  <threadedComment ref="G214" dT="2025-07-23T21:53:45.87" personId="{3DE5C77A-2EC9-410D-AF92-25A6BD2452F6}" id="{C9E6BF89-D9D3-4E3C-B697-A5DC0E655E3C}">
     <text xml:space="preserve">Converts 95% CI of the total limnetic fish estimate to a coefficient of variation, and then multiplies that by the species specific estimate to yield and SD value. 
 </text>
   </threadedComment>
-  <threadedComment ref="I213" dT="2025-07-23T21:53:45.87" personId="{3DE5C77A-2EC9-410D-AF92-25A6BD2452F6}" id="{30CBB802-82F2-45BB-8B27-7315D97962A6}">
+  <threadedComment ref="I214" dT="2025-07-23T21:53:45.87" personId="{3DE5C77A-2EC9-410D-AF92-25A6BD2452F6}" id="{30CBB802-82F2-45BB-8B27-7315D97962A6}">
     <text xml:space="preserve">Converts 95% CI of the total limnetic fish estimate to a coefficient of variation, and then multiplies that by the species specific estimate to yield and SD value. 
 </text>
   </threadedComment>
-  <threadedComment ref="G214" dT="2025-07-23T21:53:49.52" personId="{3DE5C77A-2EC9-410D-AF92-25A6BD2452F6}" id="{1FC59F05-C26A-4351-8236-C828500ADDBC}">
+  <threadedComment ref="G215" dT="2025-07-23T21:53:49.52" personId="{3DE5C77A-2EC9-410D-AF92-25A6BD2452F6}" id="{1FC59F05-C26A-4351-8236-C828500ADDBC}">
     <text xml:space="preserve">Converts 95% CI of the total limnetic fish estimate to a coefficient of variation, and then multiplies that by the species specific estimate to yield and SD value. 
 </text>
   </threadedComment>
-  <threadedComment ref="I214" dT="2025-07-23T21:53:49.52" personId="{3DE5C77A-2EC9-410D-AF92-25A6BD2452F6}" id="{1348B42C-4137-429B-A693-D62CB5C3BC03}">
+  <threadedComment ref="I215" dT="2025-07-23T21:53:49.52" personId="{3DE5C77A-2EC9-410D-AF92-25A6BD2452F6}" id="{1348B42C-4137-429B-A693-D62CB5C3BC03}">
     <text xml:space="preserve">Converts 95% CI of the total limnetic fish estimate to a coefficient of variation, and then multiplies that by the species specific estimate to yield and SD value. 
 </text>
   </threadedComment>
@@ -749,7 +767,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47CDFEE8-69FE-4C98-AD8C-E5081C486B0D}">
-  <dimension ref="A1:J313"/>
+  <dimension ref="A1:J314"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="11.7109375" bestFit="1" customWidth="1"/>
@@ -7240,7 +7258,7 @@
         <v>13</v>
       </c>
       <c r="B197">
-        <f t="shared" ref="B197:B264" si="20">YEAR(C197)</f>
+        <f t="shared" ref="B197:B265" si="20">YEAR(C197)</f>
         <v>2009</v>
       </c>
       <c r="C197" s="2">
@@ -7461,11 +7479,11 @@
         <v>40973</v>
       </c>
       <c r="D203" s="4">
-        <f t="shared" ref="D203:D270" si="21">IF(MONTH(C203)&lt;4,B203-2,B203-1)</f>
+        <f t="shared" ref="D203:D271" si="21">IF(MONTH(C203)&lt;4,B203-2,B203-1)</f>
         <v>2010</v>
       </c>
       <c r="E203" s="4">
-        <f t="shared" ref="E203:E270" si="22">IF(MONTH(C203)&lt;4,B203-3,B203-2)</f>
+        <f t="shared" ref="E203:E271" si="22">IF(MONTH(C203)&lt;4,B203-3,B203-2)</f>
         <v>2009</v>
       </c>
       <c r="F203">
@@ -7736,33 +7754,34 @@
         <v>13</v>
       </c>
       <c r="B211">
-        <f>YEAR(C211)</f>
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="C211" s="2">
-        <v>44167</v>
+        <v>43812</v>
       </c>
       <c r="D211" s="4">
-        <f>IF(MONTH(C211)&lt;4,B211-2,B211-1)</f>
-        <v>2019</v>
+        <f t="shared" si="21"/>
+        <v>2018</v>
       </c>
       <c r="E211" s="4">
-        <f>IF(MONTH(C211)&lt;4,B211-3,B211-2)</f>
-        <v>2018</v>
+        <f t="shared" si="22"/>
+        <v>2017</v>
       </c>
       <c r="F211">
-        <v>91633</v>
+        <f>943224/2</f>
+        <v>471612</v>
       </c>
       <c r="G211">
-        <f>(((1243193-976715)/1.96)/1104016)*F211</f>
-        <v>11284.487158238464</v>
+        <f>(((1046327-847837)/1.96)/943224)*F211</f>
+        <v>50635.204081632655</v>
       </c>
       <c r="H211">
-        <v>1012383</v>
+        <f>943224/2</f>
+        <v>471612</v>
       </c>
       <c r="I211">
-        <f>(((1243193-976715)/1.96)/1104016)*H211</f>
-        <v>124673.67610706766</v>
+        <f>(((1046327-847837)/1.96)/943224)*H211</f>
+        <v>50635.204081632655</v>
       </c>
       <c r="J211">
         <v>1</v>
@@ -7774,32 +7793,35 @@
       </c>
       <c r="B212">
         <f>YEAR(C212)</f>
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C212" s="2">
-        <v>44532</v>
+        <v>44167</v>
       </c>
       <c r="D212" s="4">
         <f>IF(MONTH(C212)&lt;4,B212-2,B212-1)</f>
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="E212" s="4">
         <f>IF(MONTH(C212)&lt;4,B212-3,B212-2)</f>
-        <v>2019</v>
+        <v>2018</v>
       </c>
       <c r="F212">
-        <v>28482</v>
+        <v>91633</v>
       </c>
       <c r="G212">
-        <f>(((879230-775151)/1.96)/775151)*F212</f>
-        <v>1951.1524785467077</v>
+        <f>(((1243193-976715)/1.96)/1104016)*F212</f>
+        <v>11284.487158238464</v>
       </c>
       <c r="H212">
-        <v>797496</v>
+        <v>1012383</v>
       </c>
       <c r="I212">
-        <f>(((879230-775151)/1.96)/775151)*H212</f>
-        <v>54632.269399307814</v>
+        <f>(((1243193-976715)/1.96)/1104016)*H212</f>
+        <v>124673.67610706766</v>
+      </c>
+      <c r="J212">
+        <v>1</v>
       </c>
     </row>
     <row r="213" spans="1:10" x14ac:dyDescent="0.25">
@@ -7808,10 +7830,10 @@
       </c>
       <c r="B213">
         <f>YEAR(C213)</f>
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C213" s="2">
-        <v>44615</v>
+        <v>44532</v>
       </c>
       <c r="D213" s="4">
         <f>IF(MONTH(C213)&lt;4,B213-2,B213-1)</f>
@@ -7822,21 +7844,18 @@
         <v>2019</v>
       </c>
       <c r="F213">
-        <v>17933</v>
+        <v>28482</v>
       </c>
       <c r="G213">
-        <f>(((706813-620703)/1.96)/662703)*F213</f>
-        <v>1188.8622298775329</v>
+        <f>(((879230-775151)/1.96)/775151)*F213</f>
+        <v>1951.1524785467077</v>
       </c>
       <c r="H213">
-        <v>644791</v>
+        <v>797496</v>
       </c>
       <c r="I213">
-        <f>(((706813-620703)/1.96)/662703)*H213</f>
-        <v>42746.203427478074</v>
-      </c>
-      <c r="J213">
-        <v>1</v>
+        <f>(((879230-775151)/1.96)/775151)*H213</f>
+        <v>54632.269399307814</v>
       </c>
     </row>
     <row r="214" spans="1:10" x14ac:dyDescent="0.25">
@@ -7848,29 +7867,29 @@
         <v>2022</v>
       </c>
       <c r="C214" s="2">
-        <v>44883</v>
+        <v>44615</v>
       </c>
       <c r="D214" s="4">
         <f>IF(MONTH(C214)&lt;4,B214-2,B214-1)</f>
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="E214" s="4">
         <f>IF(MONTH(C214)&lt;4,B214-3,B214-2)</f>
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="F214">
-        <v>1097034</v>
+        <v>17933</v>
       </c>
       <c r="G214">
-        <f>(((1818086-1300757)/1.96)/1706864)*F214</f>
-        <v>169641.42899146132</v>
+        <f>(((706813-620703)/1.96)/662703)*F214</f>
+        <v>1188.8622298775329</v>
       </c>
       <c r="H214">
-        <v>609830</v>
+        <v>644791</v>
       </c>
       <c r="I214">
-        <f>(((1818086-1300757)/1.96)/1706864)*H214</f>
-        <v>94301.938355477454</v>
+        <f>(((706813-620703)/1.96)/662703)*H214</f>
+        <v>42746.203427478074</v>
       </c>
       <c r="J214">
         <v>1</v>
@@ -7878,34 +7897,36 @@
     </row>
     <row r="215" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B215">
-        <f t="shared" si="20"/>
-        <v>1980</v>
+        <f>YEAR(C215)</f>
+        <v>2022</v>
       </c>
       <c r="C215" s="2">
-        <v>29277</v>
+        <v>44883</v>
       </c>
       <c r="D215" s="4">
-        <f t="shared" si="21"/>
-        <v>1978</v>
+        <f>IF(MONTH(C215)&lt;4,B215-2,B215-1)</f>
+        <v>2021</v>
       </c>
       <c r="E215" s="4">
-        <f t="shared" si="22"/>
-        <v>1977</v>
+        <f>IF(MONTH(C215)&lt;4,B215-3,B215-2)</f>
+        <v>2020</v>
       </c>
       <c r="F215">
-        <v>4623613</v>
+        <v>1097034</v>
       </c>
       <c r="G215">
-        <v>698082</v>
+        <f>(((1818086-1300757)/1.96)/1706864)*F215</f>
+        <v>169641.42899146132</v>
       </c>
       <c r="H215">
-        <v>0</v>
+        <v>609830</v>
       </c>
       <c r="I215">
-        <v>0</v>
+        <f>(((1818086-1300757)/1.96)/1706864)*H215</f>
+        <v>94301.938355477454</v>
       </c>
       <c r="J215">
         <v>1</v>
@@ -7917,30 +7938,30 @@
       </c>
       <c r="B216">
         <f t="shared" si="20"/>
-        <v>1981</v>
+        <v>1980</v>
       </c>
       <c r="C216" s="2">
-        <v>29606</v>
+        <v>29277</v>
       </c>
       <c r="D216" s="4">
         <f t="shared" si="21"/>
-        <v>1979</v>
+        <v>1978</v>
       </c>
       <c r="E216" s="4">
         <f t="shared" si="22"/>
-        <v>1978</v>
+        <v>1977</v>
       </c>
       <c r="F216">
-        <v>5684292</v>
+        <v>4623613</v>
       </c>
       <c r="G216">
-        <v>1116531</v>
+        <v>698082</v>
       </c>
       <c r="H216">
-        <v>158639</v>
+        <v>0</v>
       </c>
       <c r="I216">
-        <v>163338</v>
+        <v>0</v>
       </c>
       <c r="J216">
         <v>1</v>
@@ -7955,27 +7976,30 @@
         <v>1981</v>
       </c>
       <c r="C217" s="2">
-        <v>29803</v>
+        <v>29606</v>
       </c>
       <c r="D217" s="4">
         <f t="shared" si="21"/>
-        <v>1980</v>
+        <v>1979</v>
       </c>
       <c r="E217" s="4">
         <f t="shared" si="22"/>
-        <v>1979</v>
+        <v>1978</v>
       </c>
       <c r="F217">
-        <v>14396081</v>
+        <v>5684292</v>
       </c>
       <c r="G217">
-        <v>3293857</v>
+        <v>1116531</v>
       </c>
       <c r="H217">
-        <v>123261</v>
+        <v>158639</v>
       </c>
       <c r="I217">
-        <v>36969</v>
+        <v>163338</v>
+      </c>
+      <c r="J217">
+        <v>1</v>
       </c>
     </row>
     <row r="218" spans="1:10" x14ac:dyDescent="0.25">
@@ -7987,7 +8011,7 @@
         <v>1981</v>
       </c>
       <c r="C218" s="2">
-        <v>29858</v>
+        <v>29803</v>
       </c>
       <c r="D218" s="4">
         <f t="shared" si="21"/>
@@ -7998,16 +8022,16 @@
         <v>1979</v>
       </c>
       <c r="F218">
-        <v>11189652</v>
+        <v>14396081</v>
       </c>
       <c r="G218">
-        <v>1612712</v>
+        <v>3293857</v>
       </c>
       <c r="H218">
-        <v>0</v>
+        <v>123261</v>
       </c>
       <c r="I218">
-        <v>0</v>
+        <v>36969</v>
       </c>
     </row>
     <row r="219" spans="1:10" x14ac:dyDescent="0.25">
@@ -8019,7 +8043,7 @@
         <v>1981</v>
       </c>
       <c r="C219" s="2">
-        <v>29923</v>
+        <v>29858</v>
       </c>
       <c r="D219" s="4">
         <f t="shared" si="21"/>
@@ -8030,19 +8054,16 @@
         <v>1979</v>
       </c>
       <c r="F219">
-        <v>8335707</v>
+        <v>11189652</v>
       </c>
       <c r="G219">
-        <v>1379346</v>
+        <v>1612712</v>
       </c>
       <c r="H219">
         <v>0</v>
       </c>
       <c r="I219">
         <v>0</v>
-      </c>
-      <c r="J219">
-        <v>1</v>
       </c>
     </row>
     <row r="220" spans="1:10" x14ac:dyDescent="0.25">
@@ -8051,30 +8072,33 @@
       </c>
       <c r="B220">
         <f t="shared" si="20"/>
-        <v>1982</v>
+        <v>1981</v>
       </c>
       <c r="C220" s="2">
-        <v>30188</v>
+        <v>29923</v>
       </c>
       <c r="D220" s="4">
         <f t="shared" si="21"/>
-        <v>1981</v>
+        <v>1980</v>
       </c>
       <c r="E220" s="4">
         <f t="shared" si="22"/>
-        <v>1980</v>
+        <v>1979</v>
       </c>
       <c r="F220">
-        <v>19786826</v>
+        <v>8335707</v>
       </c>
       <c r="G220">
-        <v>3687338</v>
+        <v>1379346</v>
       </c>
       <c r="H220">
-        <v>1171047</v>
+        <v>0</v>
       </c>
       <c r="I220">
-        <v>212426</v>
+        <v>0</v>
+      </c>
+      <c r="J220">
+        <v>1</v>
       </c>
     </row>
     <row r="221" spans="1:10" x14ac:dyDescent="0.25">
@@ -8086,7 +8110,7 @@
         <v>1982</v>
       </c>
       <c r="C221" s="2">
-        <v>30265</v>
+        <v>30188</v>
       </c>
       <c r="D221" s="4">
         <f t="shared" si="21"/>
@@ -8097,16 +8121,16 @@
         <v>1980</v>
       </c>
       <c r="F221">
-        <v>7249794</v>
+        <v>19786826</v>
       </c>
       <c r="G221">
-        <v>1890346</v>
+        <v>3687338</v>
       </c>
       <c r="H221">
-        <v>435913</v>
+        <v>1171047</v>
       </c>
       <c r="I221">
-        <v>137604</v>
+        <v>212426</v>
       </c>
     </row>
     <row r="222" spans="1:10" x14ac:dyDescent="0.25">
@@ -8115,10 +8139,10 @@
       </c>
       <c r="B222">
         <f t="shared" si="20"/>
-        <v>1983</v>
+        <v>1982</v>
       </c>
       <c r="C222" s="2">
-        <v>30377</v>
+        <v>30265</v>
       </c>
       <c r="D222" s="4">
         <f t="shared" si="21"/>
@@ -8129,19 +8153,16 @@
         <v>1980</v>
       </c>
       <c r="F222">
-        <v>8427632</v>
+        <v>7249794</v>
       </c>
       <c r="G222">
-        <v>1378401</v>
+        <v>1890346</v>
       </c>
       <c r="H222">
-        <v>0</v>
+        <v>435913</v>
       </c>
       <c r="I222">
-        <v>0</v>
-      </c>
-      <c r="J222">
-        <v>1</v>
+        <v>137604</v>
       </c>
     </row>
     <row r="223" spans="1:10" x14ac:dyDescent="0.25">
@@ -8153,27 +8174,30 @@
         <v>1983</v>
       </c>
       <c r="C223" s="2">
-        <v>30551</v>
+        <v>30377</v>
       </c>
       <c r="D223" s="4">
         <f t="shared" si="21"/>
-        <v>1982</v>
+        <v>1981</v>
       </c>
       <c r="E223" s="4">
         <f t="shared" si="22"/>
-        <v>1981</v>
+        <v>1980</v>
       </c>
       <c r="F223">
-        <v>13176917</v>
+        <v>8427632</v>
       </c>
       <c r="G223">
-        <v>4038902</v>
+        <v>1378401</v>
       </c>
       <c r="H223">
-        <v>4662</v>
+        <v>0</v>
       </c>
       <c r="I223">
-        <v>5826</v>
+        <v>0</v>
+      </c>
+      <c r="J223">
+        <v>1</v>
       </c>
     </row>
     <row r="224" spans="1:10" x14ac:dyDescent="0.25">
@@ -8185,7 +8209,7 @@
         <v>1983</v>
       </c>
       <c r="C224" s="2">
-        <v>30648</v>
+        <v>30551</v>
       </c>
       <c r="D224" s="4">
         <f t="shared" si="21"/>
@@ -8196,19 +8220,16 @@
         <v>1981</v>
       </c>
       <c r="F224">
-        <v>9639172</v>
+        <v>13176917</v>
       </c>
       <c r="G224">
-        <v>1563720</v>
+        <v>4038902</v>
       </c>
       <c r="H224">
-        <v>0</v>
+        <v>4662</v>
       </c>
       <c r="I224">
-        <v>0</v>
-      </c>
-      <c r="J224">
-        <v>1</v>
+        <v>5826</v>
       </c>
     </row>
     <row r="225" spans="1:10" x14ac:dyDescent="0.25">
@@ -8217,24 +8238,24 @@
       </c>
       <c r="B225">
         <f t="shared" si="20"/>
-        <v>1984</v>
+        <v>1983</v>
       </c>
       <c r="C225" s="2">
-        <v>30956</v>
+        <v>30648</v>
       </c>
       <c r="D225" s="4">
         <f t="shared" si="21"/>
-        <v>1983</v>
+        <v>1982</v>
       </c>
       <c r="E225" s="4">
         <f t="shared" si="22"/>
-        <v>1982</v>
+        <v>1981</v>
       </c>
       <c r="F225">
-        <v>19564054</v>
+        <v>9639172</v>
       </c>
       <c r="G225">
-        <v>3521352</v>
+        <v>1563720</v>
       </c>
       <c r="H225">
         <v>0</v>
@@ -8252,24 +8273,24 @@
       </c>
       <c r="B226">
         <f t="shared" si="20"/>
-        <v>1985</v>
+        <v>1984</v>
       </c>
       <c r="C226" s="2">
-        <v>31316</v>
+        <v>30956</v>
       </c>
       <c r="D226" s="4">
         <f t="shared" si="21"/>
-        <v>1984</v>
+        <v>1983</v>
       </c>
       <c r="E226" s="4">
         <f t="shared" si="22"/>
-        <v>1983</v>
+        <v>1982</v>
       </c>
       <c r="F226">
-        <v>6970095</v>
+        <v>19564054</v>
       </c>
       <c r="G226">
-        <v>1145018</v>
+        <v>3521352</v>
       </c>
       <c r="H226">
         <v>0</v>
@@ -8290,7 +8311,7 @@
         <v>1985</v>
       </c>
       <c r="C227" s="2">
-        <v>31317</v>
+        <v>31316</v>
       </c>
       <c r="D227" s="4">
         <f t="shared" si="21"/>
@@ -8301,16 +8322,19 @@
         <v>1983</v>
       </c>
       <c r="F227">
-        <v>9079741</v>
+        <v>6970095</v>
       </c>
       <c r="G227">
-        <v>1433266</v>
+        <v>1145018</v>
       </c>
       <c r="H227">
         <v>0</v>
       </c>
       <c r="I227">
         <v>0</v>
+      </c>
+      <c r="J227">
+        <v>1</v>
       </c>
     </row>
     <row r="228" spans="1:10" x14ac:dyDescent="0.25">
@@ -8319,24 +8343,24 @@
       </c>
       <c r="B228">
         <f t="shared" si="20"/>
-        <v>1986</v>
+        <v>1985</v>
       </c>
       <c r="C228" s="2">
-        <v>31651</v>
+        <v>31317</v>
       </c>
       <c r="D228" s="4">
         <f t="shared" si="21"/>
-        <v>1985</v>
+        <v>1984</v>
       </c>
       <c r="E228" s="4">
         <f t="shared" si="22"/>
-        <v>1984</v>
+        <v>1983</v>
       </c>
       <c r="F228">
-        <v>8825549</v>
+        <v>9079741</v>
       </c>
       <c r="G228">
-        <v>2013110</v>
+        <v>1433266</v>
       </c>
       <c r="H228">
         <v>0</v>
@@ -8354,7 +8378,7 @@
         <v>1986</v>
       </c>
       <c r="C229" s="2">
-        <v>31652</v>
+        <v>31651</v>
       </c>
       <c r="D229" s="4">
         <f t="shared" si="21"/>
@@ -8365,10 +8389,10 @@
         <v>1984</v>
       </c>
       <c r="F229">
-        <v>11232287</v>
+        <v>8825549</v>
       </c>
       <c r="G229">
-        <v>2012645</v>
+        <v>2013110</v>
       </c>
       <c r="H229">
         <v>0</v>
@@ -8386,7 +8410,7 @@
         <v>1986</v>
       </c>
       <c r="C230" s="2">
-        <v>31715</v>
+        <v>31652</v>
       </c>
       <c r="D230" s="4">
         <f t="shared" si="21"/>
@@ -8397,19 +8421,16 @@
         <v>1984</v>
       </c>
       <c r="F230">
-        <v>4983068</v>
+        <v>11232287</v>
       </c>
       <c r="G230">
-        <v>114988</v>
+        <v>2012645</v>
       </c>
       <c r="H230">
-        <v>53880</v>
+        <v>0</v>
       </c>
       <c r="I230">
-        <v>23107</v>
-      </c>
-      <c r="J230">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="231" spans="1:10" x14ac:dyDescent="0.25">
@@ -8418,10 +8439,10 @@
       </c>
       <c r="B231">
         <f t="shared" si="20"/>
-        <v>1987</v>
+        <v>1986</v>
       </c>
       <c r="C231" s="2">
-        <v>31831</v>
+        <v>31715</v>
       </c>
       <c r="D231" s="4">
         <f t="shared" si="21"/>
@@ -8432,16 +8453,19 @@
         <v>1984</v>
       </c>
       <c r="F231">
-        <v>4762461</v>
+        <v>4983068</v>
       </c>
       <c r="G231">
-        <v>785400</v>
+        <v>114988</v>
       </c>
       <c r="H231">
-        <v>98338</v>
+        <v>53880</v>
       </c>
       <c r="I231">
-        <v>78489</v>
+        <v>23107</v>
+      </c>
+      <c r="J231">
+        <v>1</v>
       </c>
     </row>
     <row r="232" spans="1:10" x14ac:dyDescent="0.25">
@@ -8453,27 +8477,27 @@
         <v>1987</v>
       </c>
       <c r="C232" s="2">
-        <v>32021</v>
+        <v>31831</v>
       </c>
       <c r="D232" s="4">
         <f t="shared" si="21"/>
-        <v>1986</v>
+        <v>1985</v>
       </c>
       <c r="E232" s="4">
         <f t="shared" si="22"/>
-        <v>1985</v>
+        <v>1984</v>
       </c>
       <c r="F232">
-        <v>8560289</v>
+        <v>4762461</v>
       </c>
       <c r="G232">
-        <v>1390335</v>
+        <v>785400</v>
       </c>
       <c r="H232">
-        <v>57659</v>
+        <v>98338</v>
       </c>
       <c r="I232">
-        <v>14564</v>
+        <v>78489</v>
       </c>
     </row>
     <row r="233" spans="1:10" x14ac:dyDescent="0.25">
@@ -8485,7 +8509,7 @@
         <v>1987</v>
       </c>
       <c r="C233" s="2">
-        <v>32119</v>
+        <v>32021</v>
       </c>
       <c r="D233" s="4">
         <f t="shared" si="21"/>
@@ -8496,16 +8520,16 @@
         <v>1985</v>
       </c>
       <c r="F233">
-        <v>10840544</v>
+        <v>8560289</v>
       </c>
       <c r="G233">
-        <v>1397888</v>
+        <v>1390335</v>
       </c>
       <c r="H233">
-        <v>200451</v>
+        <v>57659</v>
       </c>
       <c r="I233">
-        <v>41137</v>
+        <v>14564</v>
       </c>
     </row>
     <row r="234" spans="1:10" x14ac:dyDescent="0.25">
@@ -8514,10 +8538,10 @@
       </c>
       <c r="B234">
         <f t="shared" si="20"/>
-        <v>1988</v>
+        <v>1987</v>
       </c>
       <c r="C234" s="2">
-        <v>32169</v>
+        <v>32119</v>
       </c>
       <c r="D234" s="4">
         <f t="shared" si="21"/>
@@ -8528,19 +8552,16 @@
         <v>1985</v>
       </c>
       <c r="F234">
-        <v>8892056</v>
+        <v>10840544</v>
       </c>
       <c r="G234">
-        <v>950613</v>
+        <v>1397888</v>
       </c>
       <c r="H234">
-        <v>0</v>
+        <v>200451</v>
       </c>
       <c r="I234">
-        <v>0</v>
-      </c>
-      <c r="J234">
-        <v>1</v>
+        <v>41137</v>
       </c>
     </row>
     <row r="235" spans="1:10" x14ac:dyDescent="0.25">
@@ -8552,21 +8573,21 @@
         <v>1988</v>
       </c>
       <c r="C235" s="2">
-        <v>32448</v>
+        <v>32169</v>
       </c>
       <c r="D235" s="4">
         <f t="shared" si="21"/>
-        <v>1987</v>
+        <v>1986</v>
       </c>
       <c r="E235" s="4">
         <f t="shared" si="22"/>
-        <v>1986</v>
+        <v>1985</v>
       </c>
       <c r="F235">
-        <v>9187558</v>
+        <v>8892056</v>
       </c>
       <c r="G235">
-        <v>1141438</v>
+        <v>950613</v>
       </c>
       <c r="H235">
         <v>0</v>
@@ -8584,30 +8605,33 @@
       </c>
       <c r="B236">
         <f t="shared" si="20"/>
-        <v>1989</v>
+        <v>1988</v>
       </c>
       <c r="C236" s="2">
-        <v>32687</v>
+        <v>32448</v>
       </c>
       <c r="D236" s="4">
         <f t="shared" si="21"/>
-        <v>1988</v>
+        <v>1987</v>
       </c>
       <c r="E236" s="4">
         <f t="shared" si="22"/>
-        <v>1987</v>
+        <v>1986</v>
       </c>
       <c r="F236">
-        <v>11813897</v>
+        <v>9187558</v>
       </c>
       <c r="G236">
-        <v>1910313</v>
+        <v>1141438</v>
       </c>
       <c r="H236">
-        <v>1923193</v>
+        <v>0</v>
       </c>
       <c r="I236">
-        <v>310981</v>
+        <v>0</v>
+      </c>
+      <c r="J236">
+        <v>1</v>
       </c>
     </row>
     <row r="237" spans="1:10" x14ac:dyDescent="0.25">
@@ -8619,7 +8643,7 @@
         <v>1989</v>
       </c>
       <c r="C237" s="2">
-        <v>32799</v>
+        <v>32687</v>
       </c>
       <c r="D237" s="4">
         <f t="shared" si="21"/>
@@ -8630,19 +8654,16 @@
         <v>1987</v>
       </c>
       <c r="F237">
-        <v>11183261</v>
+        <v>11813897</v>
       </c>
       <c r="G237">
-        <v>1959673</v>
+        <v>1910313</v>
       </c>
       <c r="H237">
-        <v>0</v>
+        <v>1923193</v>
       </c>
       <c r="I237">
-        <v>0</v>
-      </c>
-      <c r="J237">
-        <v>1</v>
+        <v>310981</v>
       </c>
     </row>
     <row r="238" spans="1:10" x14ac:dyDescent="0.25">
@@ -8654,7 +8675,7 @@
         <v>1989</v>
       </c>
       <c r="C238" s="2">
-        <v>32800</v>
+        <v>32799</v>
       </c>
       <c r="D238" s="4">
         <f t="shared" si="21"/>
@@ -8665,16 +8686,19 @@
         <v>1987</v>
       </c>
       <c r="F238">
-        <v>13224299</v>
+        <v>11183261</v>
       </c>
       <c r="G238">
-        <v>2304833</v>
+        <v>1959673</v>
       </c>
       <c r="H238">
-        <v>42305</v>
+        <v>0</v>
       </c>
       <c r="I238">
-        <v>11020</v>
+        <v>0</v>
+      </c>
+      <c r="J238">
+        <v>1</v>
       </c>
     </row>
     <row r="239" spans="1:10" x14ac:dyDescent="0.25">
@@ -8683,10 +8707,10 @@
       </c>
       <c r="B239">
         <f t="shared" si="20"/>
-        <v>1990</v>
+        <v>1989</v>
       </c>
       <c r="C239" s="2">
-        <v>32946</v>
+        <v>32800</v>
       </c>
       <c r="D239" s="4">
         <f t="shared" si="21"/>
@@ -8697,16 +8721,16 @@
         <v>1987</v>
       </c>
       <c r="F239">
-        <v>7487085</v>
+        <v>13224299</v>
       </c>
       <c r="G239">
-        <v>1092031</v>
+        <v>2304833</v>
       </c>
       <c r="H239">
-        <v>0</v>
+        <v>42305</v>
       </c>
       <c r="I239">
-        <v>0</v>
+        <v>11020</v>
       </c>
     </row>
     <row r="240" spans="1:10" x14ac:dyDescent="0.25">
@@ -8718,27 +8742,27 @@
         <v>1990</v>
       </c>
       <c r="C240" s="2">
-        <v>33035</v>
+        <v>32946</v>
       </c>
       <c r="D240" s="4">
         <f t="shared" si="21"/>
-        <v>1989</v>
+        <v>1988</v>
       </c>
       <c r="E240" s="4">
         <f t="shared" si="22"/>
-        <v>1988</v>
+        <v>1987</v>
       </c>
       <c r="F240">
-        <v>4226888</v>
+        <v>7487085</v>
       </c>
       <c r="G240">
-        <v>965642</v>
+        <v>1092031</v>
       </c>
       <c r="H240">
-        <v>1286444</v>
+        <v>0</v>
       </c>
       <c r="I240">
-        <v>293891</v>
+        <v>0</v>
       </c>
     </row>
     <row r="241" spans="1:10" x14ac:dyDescent="0.25">
@@ -8750,7 +8774,7 @@
         <v>1990</v>
       </c>
       <c r="C241" s="2">
-        <v>33036</v>
+        <v>33035</v>
       </c>
       <c r="D241" s="4">
         <f t="shared" si="21"/>
@@ -8761,16 +8785,16 @@
         <v>1988</v>
       </c>
       <c r="F241">
-        <v>4876891</v>
+        <v>4226888</v>
       </c>
       <c r="G241">
-        <v>1186063</v>
+        <v>965642</v>
       </c>
       <c r="H241">
-        <v>1484271</v>
+        <v>1286444</v>
       </c>
       <c r="I241">
-        <v>360976</v>
+        <v>293891</v>
       </c>
     </row>
     <row r="242" spans="1:10" x14ac:dyDescent="0.25">
@@ -8782,7 +8806,7 @@
         <v>1990</v>
       </c>
       <c r="C242" s="2">
-        <v>33037</v>
+        <v>33036</v>
       </c>
       <c r="D242" s="4">
         <f t="shared" si="21"/>
@@ -8793,16 +8817,16 @@
         <v>1988</v>
       </c>
       <c r="F242">
-        <v>5477969</v>
+        <v>4876891</v>
       </c>
       <c r="G242">
-        <v>1287579</v>
+        <v>1186063</v>
       </c>
       <c r="H242">
-        <v>1667208</v>
+        <v>1484271</v>
       </c>
       <c r="I242">
-        <v>391872</v>
+        <v>360976</v>
       </c>
     </row>
     <row r="243" spans="1:10" x14ac:dyDescent="0.25">
@@ -8814,7 +8838,7 @@
         <v>1990</v>
       </c>
       <c r="C243" s="2">
-        <v>33161</v>
+        <v>33037</v>
       </c>
       <c r="D243" s="4">
         <f t="shared" si="21"/>
@@ -8825,16 +8849,16 @@
         <v>1988</v>
       </c>
       <c r="F243">
-        <v>10173989</v>
+        <v>5477969</v>
       </c>
       <c r="G243">
-        <v>2119602</v>
+        <v>1287579</v>
       </c>
       <c r="H243">
-        <v>2594501</v>
+        <v>1667208</v>
       </c>
       <c r="I243">
-        <v>659443</v>
+        <v>391872</v>
       </c>
     </row>
     <row r="244" spans="1:10" x14ac:dyDescent="0.25">
@@ -8846,7 +8870,7 @@
         <v>1990</v>
       </c>
       <c r="C244" s="2">
-        <v>33162</v>
+        <v>33161</v>
       </c>
       <c r="D244" s="4">
         <f t="shared" si="21"/>
@@ -8857,16 +8881,16 @@
         <v>1988</v>
       </c>
       <c r="F244">
-        <v>9156313</v>
+        <v>10173989</v>
       </c>
       <c r="G244">
-        <v>1485174</v>
+        <v>2119602</v>
       </c>
       <c r="H244">
-        <v>2250977</v>
+        <v>2594501</v>
       </c>
       <c r="I244">
-        <v>360135</v>
+        <v>659443</v>
       </c>
     </row>
     <row r="245" spans="1:10" x14ac:dyDescent="0.25">
@@ -8878,7 +8902,7 @@
         <v>1990</v>
       </c>
       <c r="C245" s="2">
-        <v>33163</v>
+        <v>33162</v>
       </c>
       <c r="D245" s="4">
         <f t="shared" si="21"/>
@@ -8889,16 +8913,16 @@
         <v>1988</v>
       </c>
       <c r="F245">
-        <v>10967889</v>
+        <v>9156313</v>
       </c>
       <c r="G245">
-        <v>1980273</v>
+        <v>1485174</v>
       </c>
       <c r="H245">
-        <v>2706287</v>
+        <v>2250977</v>
       </c>
       <c r="I245">
-        <v>607388</v>
+        <v>360135</v>
       </c>
     </row>
     <row r="246" spans="1:10" x14ac:dyDescent="0.25">
@@ -8910,7 +8934,7 @@
         <v>1990</v>
       </c>
       <c r="C246" s="2">
-        <v>33164</v>
+        <v>33163</v>
       </c>
       <c r="D246" s="4">
         <f t="shared" si="21"/>
@@ -8921,16 +8945,16 @@
         <v>1988</v>
       </c>
       <c r="F246">
-        <v>9142123</v>
+        <v>10967889</v>
       </c>
       <c r="G246">
-        <v>1627897</v>
+        <v>1980273</v>
       </c>
       <c r="H246">
-        <v>2244214</v>
+        <v>2706287</v>
       </c>
       <c r="I246">
-        <v>445150</v>
+        <v>607388</v>
       </c>
     </row>
     <row r="247" spans="1:10" x14ac:dyDescent="0.25">
@@ -8939,10 +8963,10 @@
       </c>
       <c r="B247">
         <f t="shared" si="20"/>
-        <v>1991</v>
+        <v>1990</v>
       </c>
       <c r="C247" s="2">
-        <v>33275</v>
+        <v>33164</v>
       </c>
       <c r="D247" s="4">
         <f t="shared" si="21"/>
@@ -8953,19 +8977,16 @@
         <v>1988</v>
       </c>
       <c r="F247">
-        <v>8541187</v>
+        <v>9142123</v>
       </c>
       <c r="G247">
-        <v>1149338</v>
+        <v>1627897</v>
       </c>
       <c r="H247">
-        <v>0</v>
+        <v>2244214</v>
       </c>
       <c r="I247">
-        <v>0</v>
-      </c>
-      <c r="J247">
-        <v>1</v>
+        <v>445150</v>
       </c>
     </row>
     <row r="248" spans="1:10" x14ac:dyDescent="0.25">
@@ -8977,7 +8998,7 @@
         <v>1991</v>
       </c>
       <c r="C248" s="2">
-        <v>33278</v>
+        <v>33275</v>
       </c>
       <c r="D248" s="4">
         <f t="shared" si="21"/>
@@ -8988,16 +9009,19 @@
         <v>1988</v>
       </c>
       <c r="F248">
-        <v>8659533</v>
+        <v>8541187</v>
       </c>
       <c r="G248">
-        <v>2139007</v>
+        <v>1149338</v>
       </c>
       <c r="H248">
         <v>0</v>
       </c>
       <c r="I248">
         <v>0</v>
+      </c>
+      <c r="J248">
+        <v>1</v>
       </c>
     </row>
     <row r="249" spans="1:10" x14ac:dyDescent="0.25">
@@ -9009,21 +9033,21 @@
         <v>1991</v>
       </c>
       <c r="C249" s="2">
-        <v>33438</v>
+        <v>33278</v>
       </c>
       <c r="D249" s="4">
         <f t="shared" si="21"/>
-        <v>1990</v>
+        <v>1989</v>
       </c>
       <c r="E249" s="4">
         <f t="shared" si="22"/>
-        <v>1989</v>
+        <v>1988</v>
       </c>
       <c r="F249">
-        <v>5960245</v>
+        <v>8659533</v>
       </c>
       <c r="G249">
-        <v>1254240</v>
+        <v>2139007</v>
       </c>
       <c r="H249">
         <v>0</v>
@@ -9041,7 +9065,7 @@
         <v>1991</v>
       </c>
       <c r="C250" s="2">
-        <v>33527</v>
+        <v>33438</v>
       </c>
       <c r="D250" s="4">
         <f t="shared" si="21"/>
@@ -9052,19 +9076,16 @@
         <v>1989</v>
       </c>
       <c r="F250">
-        <v>5883006</v>
+        <v>5960245</v>
       </c>
       <c r="G250">
-        <v>1124826</v>
+        <v>1254240</v>
       </c>
       <c r="H250">
         <v>0</v>
       </c>
       <c r="I250">
         <v>0</v>
-      </c>
-      <c r="J250">
-        <v>1</v>
       </c>
     </row>
     <row r="251" spans="1:10" x14ac:dyDescent="0.25">
@@ -9073,10 +9094,10 @@
       </c>
       <c r="B251">
         <f t="shared" si="20"/>
-        <v>1992</v>
+        <v>1991</v>
       </c>
       <c r="C251" s="2">
-        <v>33658</v>
+        <v>33527</v>
       </c>
       <c r="D251" s="4">
         <f t="shared" si="21"/>
@@ -9087,16 +9108,19 @@
         <v>1989</v>
       </c>
       <c r="F251">
-        <v>4776046</v>
+        <v>5883006</v>
       </c>
       <c r="G251">
-        <v>731461</v>
+        <v>1124826</v>
       </c>
       <c r="H251">
-        <v>162138</v>
+        <v>0</v>
       </c>
       <c r="I251">
-        <v>252918</v>
+        <v>0</v>
+      </c>
+      <c r="J251">
+        <v>1</v>
       </c>
     </row>
     <row r="252" spans="1:10" x14ac:dyDescent="0.25">
@@ -9108,27 +9132,27 @@
         <v>1992</v>
       </c>
       <c r="C252" s="2">
-        <v>33798</v>
+        <v>33658</v>
       </c>
       <c r="D252" s="4">
         <f t="shared" si="21"/>
-        <v>1991</v>
+        <v>1990</v>
       </c>
       <c r="E252" s="4">
         <f t="shared" si="22"/>
-        <v>1990</v>
+        <v>1989</v>
       </c>
       <c r="F252">
-        <v>6032231</v>
+        <v>4776046</v>
       </c>
       <c r="G252">
-        <v>1248407</v>
+        <v>731461</v>
       </c>
       <c r="H252">
-        <v>0</v>
+        <v>162138</v>
       </c>
       <c r="I252">
-        <v>0</v>
+        <v>252918</v>
       </c>
     </row>
     <row r="253" spans="1:10" x14ac:dyDescent="0.25">
@@ -9140,7 +9164,7 @@
         <v>1992</v>
       </c>
       <c r="C253" s="2">
-        <v>33903</v>
+        <v>33798</v>
       </c>
       <c r="D253" s="4">
         <f t="shared" si="21"/>
@@ -9151,19 +9175,16 @@
         <v>1990</v>
       </c>
       <c r="F253">
-        <v>3372678</v>
+        <v>6032231</v>
       </c>
       <c r="G253">
-        <v>692662</v>
+        <v>1248407</v>
       </c>
       <c r="H253">
         <v>0</v>
       </c>
       <c r="I253">
         <v>0</v>
-      </c>
-      <c r="J253">
-        <v>1</v>
       </c>
     </row>
     <row r="254" spans="1:10" x14ac:dyDescent="0.25">
@@ -9172,10 +9193,10 @@
       </c>
       <c r="B254">
         <f t="shared" si="20"/>
-        <v>1993</v>
+        <v>1992</v>
       </c>
       <c r="C254" s="2">
-        <v>34010</v>
+        <v>33903</v>
       </c>
       <c r="D254" s="4">
         <f t="shared" si="21"/>
@@ -9186,16 +9207,19 @@
         <v>1990</v>
       </c>
       <c r="F254">
-        <v>4560412</v>
+        <v>3372678</v>
       </c>
       <c r="G254">
-        <v>604464</v>
+        <v>692662</v>
       </c>
       <c r="H254">
         <v>0</v>
       </c>
       <c r="I254">
         <v>0</v>
+      </c>
+      <c r="J254">
+        <v>1</v>
       </c>
     </row>
     <row r="255" spans="1:10" x14ac:dyDescent="0.25">
@@ -9207,21 +9231,21 @@
         <v>1993</v>
       </c>
       <c r="C255" s="2">
-        <v>34177</v>
+        <v>34010</v>
       </c>
       <c r="D255" s="4">
         <f t="shared" si="21"/>
-        <v>1992</v>
+        <v>1991</v>
       </c>
       <c r="E255" s="4">
         <f t="shared" si="22"/>
-        <v>1991</v>
+        <v>1990</v>
       </c>
       <c r="F255">
-        <v>10198355</v>
+        <v>4560412</v>
       </c>
       <c r="G255">
-        <v>3860607</v>
+        <v>604464</v>
       </c>
       <c r="H255">
         <v>0</v>
@@ -9239,7 +9263,7 @@
         <v>1993</v>
       </c>
       <c r="C256" s="2">
-        <v>34254</v>
+        <v>34177</v>
       </c>
       <c r="D256" s="4">
         <f t="shared" si="21"/>
@@ -9250,19 +9274,16 @@
         <v>1991</v>
       </c>
       <c r="F256">
-        <v>5992046</v>
+        <v>10198355</v>
       </c>
       <c r="G256">
-        <v>806992</v>
+        <v>3860607</v>
       </c>
       <c r="H256">
-        <v>57164</v>
+        <v>0</v>
       </c>
       <c r="I256">
-        <v>58691</v>
-      </c>
-      <c r="J256">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="257" spans="1:10" x14ac:dyDescent="0.25">
@@ -9271,10 +9292,10 @@
       </c>
       <c r="B257">
         <f t="shared" si="20"/>
-        <v>1994</v>
+        <v>1993</v>
       </c>
       <c r="C257" s="2">
-        <v>34365</v>
+        <v>34254</v>
       </c>
       <c r="D257" s="4">
         <f t="shared" si="21"/>
@@ -9285,16 +9306,19 @@
         <v>1991</v>
       </c>
       <c r="F257">
-        <v>5895395</v>
+        <v>5992046</v>
       </c>
       <c r="G257">
-        <v>780598</v>
+        <v>806992</v>
       </c>
       <c r="H257">
-        <v>0</v>
+        <v>57164</v>
       </c>
       <c r="I257">
-        <v>0</v>
+        <v>58691</v>
+      </c>
+      <c r="J257">
+        <v>1</v>
       </c>
     </row>
     <row r="258" spans="1:10" x14ac:dyDescent="0.25">
@@ -9306,27 +9330,27 @@
         <v>1994</v>
       </c>
       <c r="C258" s="2">
-        <v>34626</v>
+        <v>34365</v>
       </c>
       <c r="D258" s="4">
         <f t="shared" si="21"/>
-        <v>1993</v>
+        <v>1992</v>
       </c>
       <c r="E258" s="4">
         <f t="shared" si="22"/>
-        <v>1992</v>
+        <v>1991</v>
       </c>
       <c r="F258">
-        <v>6769766</v>
+        <v>5895395</v>
       </c>
       <c r="G258">
-        <v>732204</v>
+        <v>780598</v>
       </c>
       <c r="H258">
-        <v>109137</v>
+        <v>0</v>
       </c>
       <c r="I258">
-        <v>23773</v>
+        <v>0</v>
       </c>
     </row>
     <row r="259" spans="1:10" x14ac:dyDescent="0.25">
@@ -9335,34 +9359,30 @@
       </c>
       <c r="B259">
         <f t="shared" si="20"/>
-        <v>1995</v>
+        <v>1994</v>
       </c>
       <c r="C259" s="2">
-        <v>34730</v>
+        <v>34626</v>
       </c>
       <c r="D259" s="4">
-        <f t="shared" ref="D259" si="23">IF(MONTH(C259)&lt;4,B259-2,B259-1)</f>
+        <f t="shared" si="21"/>
         <v>1993</v>
       </c>
       <c r="E259" s="4">
-        <f t="shared" ref="E259" si="24">IF(MONTH(C259)&lt;4,B259-3,B259-2)</f>
+        <f t="shared" si="22"/>
         <v>1992</v>
       </c>
       <c r="F259">
-        <v>5895000</v>
+        <v>6769766</v>
       </c>
       <c r="G259">
-        <f>0.13*F259</f>
-        <v>766350</v>
+        <v>732204</v>
       </c>
       <c r="H259">
-        <v>0</v>
+        <v>109137</v>
       </c>
       <c r="I259">
-        <v>0</v>
-      </c>
-      <c r="J259">
-        <v>1</v>
+        <v>23773</v>
       </c>
     </row>
     <row r="260" spans="1:10" x14ac:dyDescent="0.25">
@@ -9374,27 +9394,31 @@
         <v>1995</v>
       </c>
       <c r="C260" s="2">
-        <v>34894</v>
+        <v>34730</v>
       </c>
       <c r="D260" s="4">
-        <f t="shared" si="21"/>
-        <v>1994</v>
+        <f t="shared" ref="D260" si="23">IF(MONTH(C260)&lt;4,B260-2,B260-1)</f>
+        <v>1993</v>
       </c>
       <c r="E260" s="4">
-        <f t="shared" si="22"/>
-        <v>1993</v>
+        <f t="shared" ref="E260" si="24">IF(MONTH(C260)&lt;4,B260-3,B260-2)</f>
+        <v>1992</v>
       </c>
       <c r="F260">
-        <v>10913020</v>
+        <v>5895000</v>
       </c>
       <c r="G260">
-        <v>1990404</v>
+        <f>0.13*F260</f>
+        <v>766350</v>
       </c>
       <c r="H260">
         <v>0</v>
       </c>
       <c r="I260">
         <v>0</v>
+      </c>
+      <c r="J260">
+        <v>1</v>
       </c>
     </row>
     <row r="261" spans="1:10" x14ac:dyDescent="0.25">
@@ -9406,7 +9430,7 @@
         <v>1995</v>
       </c>
       <c r="C261" s="2">
-        <v>35023</v>
+        <v>34894</v>
       </c>
       <c r="D261" s="4">
         <f t="shared" si="21"/>
@@ -9417,16 +9441,16 @@
         <v>1993</v>
       </c>
       <c r="F261">
-        <v>10634355</v>
+        <v>10913020</v>
       </c>
       <c r="G261">
-        <v>1445908</v>
+        <v>1990404</v>
       </c>
       <c r="H261">
-        <v>3462461</v>
+        <v>0</v>
       </c>
       <c r="I261">
-        <v>545953</v>
+        <v>0</v>
       </c>
     </row>
     <row r="262" spans="1:10" x14ac:dyDescent="0.25">
@@ -9438,7 +9462,7 @@
         <v>1995</v>
       </c>
       <c r="C262" s="2">
-        <v>35024</v>
+        <v>35023</v>
       </c>
       <c r="D262" s="4">
         <f t="shared" si="21"/>
@@ -9449,16 +9473,16 @@
         <v>1993</v>
       </c>
       <c r="F262">
-        <v>11699308</v>
+        <v>10634355</v>
       </c>
       <c r="G262">
-        <v>1924264</v>
+        <v>1445908</v>
       </c>
       <c r="H262">
-        <v>2394737</v>
+        <v>3462461</v>
       </c>
       <c r="I262">
-        <v>962122</v>
+        <v>545953</v>
       </c>
     </row>
     <row r="263" spans="1:10" x14ac:dyDescent="0.25">
@@ -9467,10 +9491,10 @@
       </c>
       <c r="B263">
         <f t="shared" si="20"/>
-        <v>1996</v>
+        <v>1995</v>
       </c>
       <c r="C263" s="2">
-        <v>35094</v>
+        <v>35024</v>
       </c>
       <c r="D263" s="4">
         <f t="shared" si="21"/>
@@ -9481,21 +9505,16 @@
         <v>1993</v>
       </c>
       <c r="F263">
-        <v>6152000</v>
-      </c>
-      <c r="G263" s="9">
-        <f>0.13*F263</f>
-        <v>799760</v>
+        <v>11699308</v>
+      </c>
+      <c r="G263">
+        <v>1924264</v>
       </c>
       <c r="H263">
-        <v>346000</v>
+        <v>2394737</v>
       </c>
       <c r="I263">
-        <f>0.13*H263</f>
-        <v>44980</v>
-      </c>
-      <c r="J263">
-        <v>1</v>
+        <v>962122</v>
       </c>
     </row>
     <row r="264" spans="1:10" x14ac:dyDescent="0.25">
@@ -9507,27 +9526,32 @@
         <v>1996</v>
       </c>
       <c r="C264" s="2">
-        <v>35268</v>
+        <v>35094</v>
       </c>
       <c r="D264" s="4">
         <f t="shared" si="21"/>
-        <v>1995</v>
+        <v>1994</v>
       </c>
       <c r="E264" s="4">
         <f t="shared" si="22"/>
-        <v>1994</v>
+        <v>1993</v>
       </c>
       <c r="F264">
-        <v>7258271</v>
+        <v>6152000</v>
       </c>
       <c r="G264" s="9">
-        <v>1351084</v>
+        <f>0.13*F264</f>
+        <v>799760</v>
       </c>
       <c r="H264">
-        <v>163067</v>
+        <v>346000</v>
       </c>
       <c r="I264">
-        <v>88455</v>
+        <f>0.13*H264</f>
+        <v>44980</v>
+      </c>
+      <c r="J264">
+        <v>1</v>
       </c>
     </row>
     <row r="265" spans="1:10" x14ac:dyDescent="0.25">
@@ -9535,11 +9559,11 @@
         <v>12</v>
       </c>
       <c r="B265">
-        <f t="shared" ref="B265:B312" si="25">YEAR(C265)</f>
+        <f t="shared" si="20"/>
         <v>1996</v>
       </c>
       <c r="C265" s="2">
-        <v>35388</v>
+        <v>35268</v>
       </c>
       <c r="D265" s="4">
         <f t="shared" si="21"/>
@@ -9550,16 +9574,16 @@
         <v>1994</v>
       </c>
       <c r="F265">
-        <v>4471744</v>
+        <v>7258271</v>
       </c>
       <c r="G265" s="9">
-        <v>756874</v>
+        <v>1351084</v>
       </c>
       <c r="H265">
-        <v>1083062</v>
+        <v>163067</v>
       </c>
       <c r="I265">
-        <v>253372</v>
+        <v>88455</v>
       </c>
     </row>
     <row r="266" spans="1:10" x14ac:dyDescent="0.25">
@@ -9567,11 +9591,11 @@
         <v>12</v>
       </c>
       <c r="B266">
-        <f t="shared" si="25"/>
-        <v>1997</v>
+        <f t="shared" ref="B266:B313" si="25">YEAR(C266)</f>
+        <v>1996</v>
       </c>
       <c r="C266" s="2">
-        <v>35487</v>
+        <v>35388</v>
       </c>
       <c r="D266" s="4">
         <f t="shared" si="21"/>
@@ -9582,21 +9606,16 @@
         <v>1994</v>
       </c>
       <c r="F266">
-        <v>4761000</v>
+        <v>4471744</v>
       </c>
       <c r="G266" s="9">
-        <f>0.13*F266</f>
-        <v>618930</v>
+        <v>756874</v>
       </c>
       <c r="H266">
-        <v>31000</v>
+        <v>1083062</v>
       </c>
       <c r="I266">
-        <f>0.13*H266</f>
-        <v>4030</v>
-      </c>
-      <c r="J266">
-        <v>1</v>
+        <v>253372</v>
       </c>
     </row>
     <row r="267" spans="1:10" x14ac:dyDescent="0.25">
@@ -9608,29 +9627,29 @@
         <v>1997</v>
       </c>
       <c r="C267" s="2">
-        <v>35753</v>
+        <v>35487</v>
       </c>
       <c r="D267" s="4">
         <f t="shared" si="21"/>
-        <v>1996</v>
+        <v>1995</v>
       </c>
       <c r="E267" s="4">
         <f t="shared" si="22"/>
-        <v>1995</v>
+        <v>1994</v>
       </c>
       <c r="F267">
-        <v>18123000</v>
+        <v>4761000</v>
       </c>
       <c r="G267" s="9">
         <f>0.13*F267</f>
-        <v>2355990</v>
+        <v>618930</v>
       </c>
       <c r="H267">
-        <v>648000</v>
+        <v>31000</v>
       </c>
       <c r="I267">
         <f>0.13*H267</f>
-        <v>84240</v>
+        <v>4030</v>
       </c>
       <c r="J267">
         <v>1</v>
@@ -9642,10 +9661,10 @@
       </c>
       <c r="B268">
         <f t="shared" si="25"/>
-        <v>1998</v>
+        <v>1997</v>
       </c>
       <c r="C268" s="2">
-        <v>35859</v>
+        <v>35753</v>
       </c>
       <c r="D268" s="4">
         <f t="shared" si="21"/>
@@ -9656,18 +9675,21 @@
         <v>1995</v>
       </c>
       <c r="F268">
-        <v>8515000</v>
+        <v>18123000</v>
       </c>
       <c r="G268" s="9">
-        <f>0.18*F268</f>
-        <v>1532700</v>
+        <f>0.13*F268</f>
+        <v>2355990</v>
       </c>
       <c r="H268">
-        <v>49000</v>
+        <v>648000</v>
       </c>
       <c r="I268">
-        <f>0.18*H268</f>
-        <v>8820</v>
+        <f>0.13*H268</f>
+        <v>84240</v>
+      </c>
+      <c r="J268">
+        <v>1</v>
       </c>
     </row>
     <row r="269" spans="1:10" x14ac:dyDescent="0.25">
@@ -9679,29 +9701,29 @@
         <v>1998</v>
       </c>
       <c r="C269" s="2">
-        <v>36007</v>
+        <v>35859</v>
       </c>
       <c r="D269" s="4">
         <f t="shared" si="21"/>
-        <v>1997</v>
+        <v>1996</v>
       </c>
       <c r="E269" s="4">
         <f t="shared" si="22"/>
-        <v>1996</v>
+        <v>1995</v>
       </c>
       <c r="F269">
-        <v>9573000</v>
+        <v>8515000</v>
       </c>
       <c r="G269" s="9">
-        <f>0.24*F269</f>
-        <v>2297520</v>
+        <f>0.18*F269</f>
+        <v>1532700</v>
       </c>
       <c r="H269">
-        <v>22000</v>
+        <v>49000</v>
       </c>
       <c r="I269">
-        <f>0.24*H269</f>
-        <v>5280</v>
+        <f>0.18*H269</f>
+        <v>8820</v>
       </c>
     </row>
     <row r="270" spans="1:10" x14ac:dyDescent="0.25">
@@ -9713,7 +9735,7 @@
         <v>1998</v>
       </c>
       <c r="C270" s="2">
-        <v>36130</v>
+        <v>36007</v>
       </c>
       <c r="D270" s="4">
         <f t="shared" si="21"/>
@@ -9724,20 +9746,18 @@
         <v>1996</v>
       </c>
       <c r="F270">
-        <v>8233000</v>
+        <v>9573000</v>
       </c>
       <c r="G270" s="9">
-        <f>0.09*F270</f>
-        <v>740970</v>
+        <f>0.24*F270</f>
+        <v>2297520</v>
       </c>
       <c r="H270">
-        <v>0</v>
+        <v>22000</v>
       </c>
       <c r="I270">
-        <v>0</v>
-      </c>
-      <c r="J270">
-        <v>1</v>
+        <f>0.24*H270</f>
+        <v>5280</v>
       </c>
     </row>
     <row r="271" spans="1:10" x14ac:dyDescent="0.25">
@@ -9746,25 +9766,34 @@
       </c>
       <c r="B271">
         <f t="shared" si="25"/>
-        <v>1999</v>
+        <v>1998</v>
       </c>
       <c r="C271" s="2">
-        <v>36338</v>
+        <v>36130</v>
       </c>
       <c r="D271" s="4">
-        <f t="shared" ref="D271:D272" si="26">IF(MONTH(C271)&lt;4,B271-2,B271-1)</f>
-        <v>1998</v>
+        <f t="shared" si="21"/>
+        <v>1997</v>
       </c>
       <c r="E271" s="4">
-        <f t="shared" ref="E271:E272" si="27">IF(MONTH(C271)&lt;4,B271-3,B271-2)</f>
-        <v>1997</v>
+        <f t="shared" si="22"/>
+        <v>1996</v>
       </c>
       <c r="F271">
-        <v>5386000</v>
+        <v>8233000</v>
       </c>
       <c r="G271" s="9">
-        <f>0.29*F271</f>
-        <v>1561940</v>
+        <f>0.09*F271</f>
+        <v>740970</v>
+      </c>
+      <c r="H271">
+        <v>0</v>
+      </c>
+      <c r="I271">
+        <v>0</v>
+      </c>
+      <c r="J271">
+        <v>1</v>
       </c>
     </row>
     <row r="272" spans="1:10" x14ac:dyDescent="0.25">
@@ -9776,22 +9805,22 @@
         <v>1999</v>
       </c>
       <c r="C272" s="2">
-        <v>36362</v>
+        <v>36338</v>
       </c>
       <c r="D272" s="4">
-        <f t="shared" si="26"/>
+        <f t="shared" ref="D272:D273" si="26">IF(MONTH(C272)&lt;4,B272-2,B272-1)</f>
         <v>1998</v>
       </c>
       <c r="E272" s="4">
-        <f t="shared" si="27"/>
+        <f t="shared" ref="E272:E273" si="27">IF(MONTH(C272)&lt;4,B272-3,B272-2)</f>
         <v>1997</v>
       </c>
       <c r="F272">
-        <v>7141000</v>
+        <v>5386000</v>
       </c>
       <c r="G272" s="9">
-        <f>0.25*F272</f>
-        <v>1785250</v>
+        <f>0.29*F272</f>
+        <v>1561940</v>
       </c>
     </row>
     <row r="273" spans="1:10" x14ac:dyDescent="0.25">
@@ -9803,31 +9832,22 @@
         <v>1999</v>
       </c>
       <c r="C273" s="2">
-        <v>36494</v>
+        <v>36362</v>
       </c>
       <c r="D273" s="4">
-        <f t="shared" ref="D273:D312" si="28">IF(MONTH(C273)&lt;4,B273-2,B273-1)</f>
+        <f t="shared" si="26"/>
         <v>1998</v>
       </c>
       <c r="E273" s="4">
-        <f t="shared" ref="E273:E312" si="29">IF(MONTH(C273)&lt;4,B273-3,B273-2)</f>
+        <f t="shared" si="27"/>
         <v>1997</v>
       </c>
       <c r="F273">
-        <v>8462000</v>
+        <v>7141000</v>
       </c>
       <c r="G273" s="9">
-        <f>0.12*F273</f>
-        <v>1015440</v>
-      </c>
-      <c r="H273">
-        <v>0</v>
-      </c>
-      <c r="I273">
-        <v>0</v>
-      </c>
-      <c r="J273">
-        <v>1</v>
+        <f>0.25*F273</f>
+        <v>1785250</v>
       </c>
     </row>
     <row r="274" spans="1:10" x14ac:dyDescent="0.25">
@@ -9836,25 +9856,25 @@
       </c>
       <c r="B274">
         <f t="shared" si="25"/>
-        <v>2000</v>
+        <v>1999</v>
       </c>
       <c r="C274" s="2">
-        <v>36858</v>
+        <v>36494</v>
       </c>
       <c r="D274" s="4">
-        <f t="shared" si="28"/>
-        <v>1999</v>
+        <f t="shared" ref="D274:D313" si="28">IF(MONTH(C274)&lt;4,B274-2,B274-1)</f>
+        <v>1998</v>
       </c>
       <c r="E274" s="4">
-        <f t="shared" si="29"/>
-        <v>1998</v>
+        <f t="shared" ref="E274:E313" si="29">IF(MONTH(C274)&lt;4,B274-3,B274-2)</f>
+        <v>1997</v>
       </c>
       <c r="F274">
-        <v>9679000</v>
+        <v>8462000</v>
       </c>
       <c r="G274" s="9">
-        <f>0.15*F274</f>
-        <v>1451850</v>
+        <f>0.12*F274</f>
+        <v>1015440</v>
       </c>
       <c r="H274">
         <v>0</v>
@@ -9872,32 +9892,31 @@
       </c>
       <c r="B275">
         <f t="shared" si="25"/>
-        <v>2001</v>
+        <v>2000</v>
       </c>
       <c r="C275" s="2">
-        <v>37230</v>
+        <v>36858</v>
       </c>
       <c r="D275" s="4">
         <f t="shared" si="28"/>
-        <v>2000</v>
+        <v>1999</v>
       </c>
       <c r="E275" s="4">
         <f t="shared" si="29"/>
-        <v>1999</v>
+        <v>1998</v>
       </c>
       <c r="F275">
-        <v>7478000</v>
+        <v>9679000</v>
       </c>
       <c r="G275" s="9">
-        <f>0.14*F275</f>
-        <v>1046920.0000000001</v>
+        <f>0.15*F275</f>
+        <v>1451850</v>
       </c>
       <c r="H275">
-        <v>326000</v>
+        <v>0</v>
       </c>
       <c r="I275">
-        <f>0.14*H275</f>
-        <v>45640.000000000007</v>
+        <v>0</v>
       </c>
       <c r="J275">
         <v>1</v>
@@ -9908,51 +9927,52 @@
         <v>12</v>
       </c>
       <c r="B276">
-        <v>2002</v>
+        <f t="shared" si="25"/>
+        <v>2001</v>
+      </c>
+      <c r="C276" s="2">
+        <v>37230</v>
       </c>
       <c r="D276" s="4">
-        <v>2001</v>
+        <f t="shared" si="28"/>
+        <v>2000</v>
       </c>
       <c r="E276" s="4">
-        <v>2000</v>
-      </c>
-      <c r="G276" s="9"/>
+        <f t="shared" si="29"/>
+        <v>1999</v>
+      </c>
+      <c r="F276">
+        <v>7478000</v>
+      </c>
+      <c r="G276" s="9">
+        <f>0.14*F276</f>
+        <v>1046920.0000000001</v>
+      </c>
+      <c r="H276">
+        <v>326000</v>
+      </c>
+      <c r="I276">
+        <f>0.14*H276</f>
+        <v>45640.000000000007</v>
+      </c>
+      <c r="J276">
+        <v>1</v>
+      </c>
     </row>
     <row r="277" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A277" t="s">
         <v>12</v>
       </c>
       <c r="B277">
-        <f t="shared" si="25"/>
-        <v>2003</v>
-      </c>
-      <c r="C277" s="2">
-        <v>37637</v>
+        <v>2002</v>
       </c>
       <c r="D277" s="4">
-        <f t="shared" si="28"/>
         <v>2001</v>
       </c>
       <c r="E277" s="4">
-        <f t="shared" si="29"/>
         <v>2000</v>
       </c>
-      <c r="F277">
-        <v>4773000</v>
-      </c>
-      <c r="G277" s="9">
-        <f>0.16*F277</f>
-        <v>763680</v>
-      </c>
-      <c r="H277">
-        <v>0</v>
-      </c>
-      <c r="I277">
-        <v>0</v>
-      </c>
-      <c r="J277">
-        <v>1</v>
-      </c>
+      <c r="G277" s="9"/>
     </row>
     <row r="278" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A278" t="s">
@@ -9960,24 +9980,25 @@
       </c>
       <c r="B278">
         <f t="shared" si="25"/>
-        <v>2004</v>
+        <v>2003</v>
       </c>
       <c r="C278" s="2">
-        <v>38005</v>
+        <v>37637</v>
       </c>
       <c r="D278" s="4">
         <f t="shared" si="28"/>
-        <v>2002</v>
+        <v>2001</v>
       </c>
       <c r="E278" s="4">
         <f t="shared" si="29"/>
-        <v>2001</v>
+        <v>2000</v>
       </c>
       <c r="F278">
-        <v>8636807</v>
+        <v>4773000</v>
       </c>
       <c r="G278" s="9">
-        <v>1694839</v>
+        <f>0.16*F278</f>
+        <v>763680</v>
       </c>
       <c r="H278">
         <v>0</v>
@@ -9995,24 +10016,24 @@
       </c>
       <c r="B279">
         <f t="shared" si="25"/>
-        <v>2005</v>
+        <v>2004</v>
       </c>
       <c r="C279" s="2">
-        <v>38378</v>
+        <v>38005</v>
       </c>
       <c r="D279" s="4">
         <f t="shared" si="28"/>
-        <v>2003</v>
+        <v>2002</v>
       </c>
       <c r="E279" s="4">
         <f t="shared" si="29"/>
-        <v>2002</v>
+        <v>2001</v>
       </c>
       <c r="F279">
-        <v>6703046</v>
+        <v>8636807</v>
       </c>
       <c r="G279" s="9">
-        <v>1052271</v>
+        <v>1694839</v>
       </c>
       <c r="H279">
         <v>0</v>
@@ -10030,24 +10051,24 @@
       </c>
       <c r="B280">
         <f t="shared" si="25"/>
-        <v>2006</v>
+        <v>2005</v>
       </c>
       <c r="C280" s="2">
-        <v>38721</v>
+        <v>38378</v>
       </c>
       <c r="D280" s="4">
         <f t="shared" si="28"/>
-        <v>2004</v>
+        <v>2003</v>
       </c>
       <c r="E280" s="4">
         <f t="shared" si="29"/>
-        <v>2003</v>
+        <v>2002</v>
       </c>
       <c r="F280">
-        <v>3525291</v>
-      </c>
-      <c r="G280">
-        <v>719392</v>
+        <v>6703046</v>
+      </c>
+      <c r="G280" s="9">
+        <v>1052271</v>
       </c>
       <c r="H280">
         <v>0</v>
@@ -10065,25 +10086,24 @@
       </c>
       <c r="B281">
         <f t="shared" si="25"/>
-        <v>2007</v>
+        <v>2006</v>
       </c>
       <c r="C281" s="2">
-        <v>39120</v>
+        <v>38721</v>
       </c>
       <c r="D281" s="4">
         <f t="shared" si="28"/>
-        <v>2005</v>
+        <v>2004</v>
       </c>
       <c r="E281" s="4">
         <f t="shared" si="29"/>
-        <v>2004</v>
+        <v>2003</v>
       </c>
       <c r="F281">
-        <v>3660000</v>
+        <v>3525291</v>
       </c>
       <c r="G281">
-        <f>0.14*F281</f>
-        <v>512400.00000000006</v>
+        <v>719392</v>
       </c>
       <c r="H281">
         <v>0</v>
@@ -10104,29 +10124,28 @@
         <v>2007</v>
       </c>
       <c r="C282" s="2">
-        <v>39395</v>
+        <v>39120</v>
       </c>
       <c r="D282" s="4">
         <f t="shared" si="28"/>
-        <v>2006</v>
+        <v>2005</v>
       </c>
       <c r="E282" s="4">
         <f t="shared" si="29"/>
-        <v>2005</v>
+        <v>2004</v>
       </c>
       <c r="F282">
-        <v>5048000</v>
+        <v>3660000</v>
       </c>
       <c r="G282">
-        <f>0.18*F282</f>
-        <v>908640</v>
+        <f>0.14*F282</f>
+        <v>512400.00000000006</v>
       </c>
       <c r="H282">
-        <v>51000</v>
+        <v>0</v>
       </c>
       <c r="I282">
-        <f>0.18*H282</f>
-        <v>9180</v>
+        <v>0</v>
       </c>
       <c r="J282">
         <v>1</v>
@@ -10138,31 +10157,35 @@
       </c>
       <c r="B283">
         <f t="shared" si="25"/>
-        <v>2008</v>
+        <v>2007</v>
       </c>
       <c r="C283" s="2">
-        <v>39651</v>
+        <v>39395</v>
       </c>
       <c r="D283" s="4">
         <f t="shared" si="28"/>
-        <v>2007</v>
+        <v>2006</v>
       </c>
       <c r="E283" s="4">
         <f t="shared" si="29"/>
-        <v>2006</v>
+        <v>2005</v>
       </c>
       <c r="F283">
-        <v>5541000</v>
+        <v>5048000</v>
       </c>
       <c r="G283">
-        <f>0.28*F283</f>
-        <v>1551480.0000000002</v>
+        <f>0.18*F283</f>
+        <v>908640</v>
       </c>
       <c r="H283">
-        <v>0</v>
+        <v>51000</v>
       </c>
       <c r="I283">
-        <v>0</v>
+        <f>0.18*H283</f>
+        <v>9180</v>
+      </c>
+      <c r="J283">
+        <v>1</v>
       </c>
     </row>
     <row r="284" spans="1:10" x14ac:dyDescent="0.25">
@@ -10174,7 +10197,7 @@
         <v>2008</v>
       </c>
       <c r="C284" s="2">
-        <v>39769</v>
+        <v>39651</v>
       </c>
       <c r="D284" s="4">
         <f t="shared" si="28"/>
@@ -10185,20 +10208,17 @@
         <v>2006</v>
       </c>
       <c r="F284">
-        <v>6017000</v>
+        <v>5541000</v>
       </c>
       <c r="G284">
-        <f>0.16*F284</f>
-        <v>962720</v>
+        <f>0.28*F284</f>
+        <v>1551480.0000000002</v>
       </c>
       <c r="H284">
         <v>0</v>
       </c>
       <c r="I284">
         <v>0</v>
-      </c>
-      <c r="J284">
-        <v>1</v>
       </c>
     </row>
     <row r="285" spans="1:10" x14ac:dyDescent="0.25">
@@ -10210,7 +10230,7 @@
         <v>2008</v>
       </c>
       <c r="C285" s="2">
-        <v>39783</v>
+        <v>39769</v>
       </c>
       <c r="D285" s="4">
         <f t="shared" si="28"/>
@@ -10221,16 +10241,20 @@
         <v>2006</v>
       </c>
       <c r="F285">
-        <v>6017335</v>
+        <v>6017000</v>
       </c>
       <c r="G285">
-        <v>935967</v>
+        <f>0.16*F285</f>
+        <v>962720</v>
       </c>
       <c r="H285">
         <v>0</v>
       </c>
       <c r="I285">
         <v>0</v>
+      </c>
+      <c r="J285">
+        <v>1</v>
       </c>
     </row>
     <row r="286" spans="1:10" x14ac:dyDescent="0.25">
@@ -10239,25 +10263,24 @@
       </c>
       <c r="B286">
         <f t="shared" si="25"/>
-        <v>2009</v>
+        <v>2008</v>
       </c>
       <c r="C286" s="2">
-        <v>39973</v>
+        <v>39783</v>
       </c>
       <c r="D286" s="4">
         <f t="shared" si="28"/>
-        <v>2008</v>
+        <v>2007</v>
       </c>
       <c r="E286" s="4">
         <f t="shared" si="29"/>
-        <v>2007</v>
+        <v>2006</v>
       </c>
       <c r="F286">
-        <v>5540818</v>
+        <v>6017335</v>
       </c>
       <c r="G286">
-        <f>0.28*F286</f>
-        <v>1551429.04</v>
+        <v>935967</v>
       </c>
       <c r="H286">
         <v>0</v>
@@ -10275,7 +10298,7 @@
         <v>2009</v>
       </c>
       <c r="C287" s="2">
-        <v>40049</v>
+        <v>39973</v>
       </c>
       <c r="D287" s="4">
         <f t="shared" si="28"/>
@@ -10286,11 +10309,11 @@
         <v>2007</v>
       </c>
       <c r="F287">
-        <v>7596484</v>
+        <v>5540818</v>
       </c>
       <c r="G287">
-        <f>0.2*F287</f>
-        <v>1519296.8</v>
+        <f>0.28*F287</f>
+        <v>1551429.04</v>
       </c>
       <c r="H287">
         <v>0</v>
@@ -10308,7 +10331,7 @@
         <v>2009</v>
       </c>
       <c r="C288" s="2">
-        <v>40147</v>
+        <v>40049</v>
       </c>
       <c r="D288" s="4">
         <f t="shared" si="28"/>
@@ -10319,20 +10342,17 @@
         <v>2007</v>
       </c>
       <c r="F288">
-        <v>2450742</v>
+        <v>7596484</v>
       </c>
       <c r="G288">
-        <f>0.19*F288</f>
-        <v>465640.98</v>
+        <f>0.2*F288</f>
+        <v>1519296.8</v>
       </c>
       <c r="H288">
         <v>0</v>
       </c>
       <c r="I288">
         <v>0</v>
-      </c>
-      <c r="J288">
-        <v>1</v>
       </c>
     </row>
     <row r="289" spans="1:10" x14ac:dyDescent="0.25">
@@ -10341,10 +10361,10 @@
       </c>
       <c r="B289">
         <f t="shared" si="25"/>
-        <v>2010</v>
+        <v>2009</v>
       </c>
       <c r="C289" s="2">
-        <v>40191</v>
+        <v>40147</v>
       </c>
       <c r="D289" s="4">
         <f t="shared" si="28"/>
@@ -10355,17 +10375,20 @@
         <v>2007</v>
       </c>
       <c r="F289">
-        <v>4979378</v>
+        <v>2450742</v>
       </c>
       <c r="G289">
-        <f>0.12*F289</f>
-        <v>597525.36</v>
+        <f>0.19*F289</f>
+        <v>465640.98</v>
       </c>
       <c r="H289">
         <v>0</v>
       </c>
       <c r="I289">
         <v>0</v>
+      </c>
+      <c r="J289">
+        <v>1</v>
       </c>
     </row>
     <row r="290" spans="1:10" x14ac:dyDescent="0.25">
@@ -10377,21 +10400,22 @@
         <v>2010</v>
       </c>
       <c r="C290" s="2">
-        <v>40406</v>
+        <v>40191</v>
       </c>
       <c r="D290" s="4">
         <f t="shared" si="28"/>
-        <v>2009</v>
+        <v>2008</v>
       </c>
       <c r="E290" s="4">
         <f t="shared" si="29"/>
-        <v>2008</v>
+        <v>2007</v>
       </c>
       <c r="F290">
-        <v>16661391</v>
+        <v>4979378</v>
       </c>
       <c r="G290">
-        <v>5621822</v>
+        <f>0.12*F290</f>
+        <v>597525.36</v>
       </c>
       <c r="H290">
         <v>0</v>
@@ -10409,7 +10433,7 @@
         <v>2010</v>
       </c>
       <c r="C291" s="2">
-        <v>40414</v>
+        <v>40406</v>
       </c>
       <c r="D291" s="4">
         <f t="shared" si="28"/>
@@ -10420,10 +10444,10 @@
         <v>2008</v>
       </c>
       <c r="F291">
-        <v>8166458</v>
+        <v>16661391</v>
       </c>
       <c r="G291">
-        <v>2639773</v>
+        <v>5621822</v>
       </c>
       <c r="H291">
         <v>0</v>
@@ -10441,7 +10465,7 @@
         <v>2010</v>
       </c>
       <c r="C292" s="2">
-        <v>40512</v>
+        <v>40414</v>
       </c>
       <c r="D292" s="4">
         <f t="shared" si="28"/>
@@ -10452,20 +10476,16 @@
         <v>2008</v>
       </c>
       <c r="F292">
-        <v>14526189</v>
+        <v>8166458</v>
       </c>
       <c r="G292">
-        <f>0.24*F292</f>
-        <v>3486285.36</v>
+        <v>2639773</v>
       </c>
       <c r="H292">
         <v>0</v>
       </c>
       <c r="I292">
         <v>0</v>
-      </c>
-      <c r="J292">
-        <v>1</v>
       </c>
     </row>
     <row r="293" spans="1:10" x14ac:dyDescent="0.25">
@@ -10474,31 +10494,34 @@
       </c>
       <c r="B293">
         <f t="shared" si="25"/>
-        <v>2011</v>
+        <v>2010</v>
       </c>
       <c r="C293" s="2">
-        <v>40771</v>
+        <v>40512</v>
       </c>
       <c r="D293" s="4">
         <f t="shared" si="28"/>
-        <v>2010</v>
+        <v>2009</v>
       </c>
       <c r="E293" s="4">
         <f t="shared" si="29"/>
-        <v>2009</v>
+        <v>2008</v>
       </c>
       <c r="F293">
-        <v>16661391</v>
+        <v>14526189</v>
       </c>
       <c r="G293">
-        <f>0.34*F293</f>
-        <v>5664872.9400000004</v>
+        <f>0.24*F293</f>
+        <v>3486285.36</v>
       </c>
       <c r="H293">
         <v>0</v>
       </c>
       <c r="I293">
         <v>0</v>
+      </c>
+      <c r="J293">
+        <v>1</v>
       </c>
     </row>
     <row r="294" spans="1:10" x14ac:dyDescent="0.25">
@@ -10510,7 +10533,7 @@
         <v>2011</v>
       </c>
       <c r="C294" s="2">
-        <v>40868</v>
+        <v>40771</v>
       </c>
       <c r="D294" s="4">
         <f t="shared" si="28"/>
@@ -10521,20 +10544,17 @@
         <v>2009</v>
       </c>
       <c r="F294">
-        <v>13444391</v>
+        <v>16661391</v>
       </c>
       <c r="G294">
-        <f>0.09*F294</f>
-        <v>1209995.19</v>
+        <f>0.34*F294</f>
+        <v>5664872.9400000004</v>
       </c>
       <c r="H294">
         <v>0</v>
       </c>
       <c r="I294">
         <v>0</v>
-      </c>
-      <c r="J294">
-        <v>1</v>
       </c>
     </row>
     <row r="295" spans="1:10" x14ac:dyDescent="0.25">
@@ -10543,30 +10563,34 @@
       </c>
       <c r="B295">
         <f t="shared" si="25"/>
-        <v>2012</v>
+        <v>2011</v>
       </c>
       <c r="C295" s="2">
-        <v>41226</v>
+        <v>40868</v>
       </c>
       <c r="D295" s="4">
         <f t="shared" si="28"/>
-        <v>2011</v>
+        <v>2010</v>
       </c>
       <c r="E295" s="4">
         <f t="shared" si="29"/>
-        <v>2010</v>
+        <v>2009</v>
       </c>
       <c r="F295">
-        <v>14526189</v>
+        <v>13444391</v>
       </c>
       <c r="G295">
-        <v>2099030</v>
+        <f>0.09*F295</f>
+        <v>1209995.19</v>
       </c>
       <c r="H295">
-        <v>14526189</v>
+        <v>0</v>
       </c>
       <c r="I295">
-        <v>2099030</v>
+        <v>0</v>
+      </c>
+      <c r="J295">
+        <v>1</v>
       </c>
     </row>
     <row r="296" spans="1:10" x14ac:dyDescent="0.25">
@@ -10578,7 +10602,7 @@
         <v>2012</v>
       </c>
       <c r="C296" s="2">
-        <v>41073</v>
+        <v>41226</v>
       </c>
       <c r="D296" s="4">
         <f t="shared" si="28"/>
@@ -10589,16 +10613,16 @@
         <v>2010</v>
       </c>
       <c r="F296">
-        <v>15262441</v>
+        <v>14526189</v>
       </c>
       <c r="G296">
-        <v>5573233</v>
+        <v>2099030</v>
       </c>
       <c r="H296">
-        <v>0</v>
+        <v>14526189</v>
       </c>
       <c r="I296">
-        <v>0</v>
+        <v>2099030</v>
       </c>
     </row>
     <row r="297" spans="1:10" x14ac:dyDescent="0.25">
@@ -10610,7 +10634,7 @@
         <v>2012</v>
       </c>
       <c r="C297" s="2">
-        <v>41136</v>
+        <v>41073</v>
       </c>
       <c r="D297" s="4">
         <f t="shared" si="28"/>
@@ -10621,10 +10645,10 @@
         <v>2010</v>
       </c>
       <c r="F297">
-        <v>21862120</v>
+        <v>15262441</v>
       </c>
       <c r="G297">
-        <v>7651741.9999999991</v>
+        <v>5573233</v>
       </c>
       <c r="H297">
         <v>0</v>
@@ -10639,10 +10663,10 @@
       </c>
       <c r="B298">
         <f t="shared" si="25"/>
-        <v>2013</v>
+        <v>2012</v>
       </c>
       <c r="C298" s="2">
-        <v>41331</v>
+        <v>41136</v>
       </c>
       <c r="D298" s="4">
         <f t="shared" si="28"/>
@@ -10653,20 +10677,16 @@
         <v>2010</v>
       </c>
       <c r="F298">
-        <v>14526189</v>
+        <v>21862120</v>
       </c>
       <c r="G298">
-        <f>0.14*F298</f>
-        <v>2033666.4600000002</v>
+        <v>7651741.9999999991</v>
       </c>
       <c r="H298">
         <v>0</v>
       </c>
       <c r="I298">
         <v>0</v>
-      </c>
-      <c r="J298">
-        <v>1</v>
       </c>
     </row>
     <row r="299" spans="1:10" x14ac:dyDescent="0.25">
@@ -10678,28 +10698,31 @@
         <v>2013</v>
       </c>
       <c r="C299" s="2">
-        <v>41513</v>
+        <v>41331</v>
       </c>
       <c r="D299" s="4">
         <f t="shared" si="28"/>
-        <v>2012</v>
+        <v>2011</v>
       </c>
       <c r="E299" s="4">
         <f t="shared" si="29"/>
-        <v>2011</v>
+        <v>2010</v>
       </c>
       <c r="F299">
-        <v>11210000</v>
+        <v>14526189</v>
       </c>
       <c r="G299">
-        <f>0.21*F299</f>
-        <v>2354100</v>
+        <f>0.14*F299</f>
+        <v>2033666.4600000002</v>
       </c>
       <c r="H299">
         <v>0</v>
       </c>
       <c r="I299">
         <v>0</v>
+      </c>
+      <c r="J299">
+        <v>1</v>
       </c>
     </row>
     <row r="300" spans="1:10" x14ac:dyDescent="0.25">
@@ -10711,7 +10734,7 @@
         <v>2013</v>
       </c>
       <c r="C300" s="2">
-        <v>41597</v>
+        <v>41513</v>
       </c>
       <c r="D300" s="4">
         <f t="shared" si="28"/>
@@ -10722,20 +10745,17 @@
         <v>2011</v>
       </c>
       <c r="F300">
-        <v>3687000</v>
+        <v>11210000</v>
       </c>
       <c r="G300">
-        <f>0.31*F300</f>
-        <v>1142970</v>
+        <f>0.21*F300</f>
+        <v>2354100</v>
       </c>
       <c r="H300">
         <v>0</v>
       </c>
       <c r="I300">
         <v>0</v>
-      </c>
-      <c r="J300">
-        <v>1</v>
       </c>
     </row>
     <row r="301" spans="1:10" x14ac:dyDescent="0.25">
@@ -10744,31 +10764,34 @@
       </c>
       <c r="B301">
         <f t="shared" si="25"/>
-        <v>2014</v>
+        <v>2013</v>
       </c>
       <c r="C301" s="2">
-        <v>41932</v>
+        <v>41597</v>
       </c>
       <c r="D301" s="4">
         <f t="shared" si="28"/>
-        <v>2013</v>
+        <v>2012</v>
       </c>
       <c r="E301" s="4">
         <f t="shared" si="29"/>
-        <v>2012</v>
+        <v>2011</v>
       </c>
       <c r="F301">
-        <v>13157290</v>
+        <v>3687000</v>
       </c>
       <c r="G301">
-        <f>0.28*F301</f>
-        <v>3684041.2</v>
+        <f>0.31*F301</f>
+        <v>1142970</v>
       </c>
       <c r="H301">
         <v>0</v>
       </c>
       <c r="I301">
         <v>0</v>
+      </c>
+      <c r="J301">
+        <v>1</v>
       </c>
     </row>
     <row r="302" spans="1:10" x14ac:dyDescent="0.25">
@@ -10777,10 +10800,10 @@
       </c>
       <c r="B302">
         <f t="shared" si="25"/>
-        <v>2015</v>
+        <v>2014</v>
       </c>
       <c r="C302" s="2">
-        <v>42042</v>
+        <v>41932</v>
       </c>
       <c r="D302" s="4">
         <f t="shared" si="28"/>
@@ -10791,20 +10814,17 @@
         <v>2012</v>
       </c>
       <c r="F302">
-        <v>1210757</v>
+        <v>13157290</v>
       </c>
       <c r="G302">
-        <f>F302*0.23</f>
-        <v>278474.11</v>
+        <f>0.28*F302</f>
+        <v>3684041.2</v>
       </c>
       <c r="H302">
         <v>0</v>
       </c>
       <c r="I302">
         <v>0</v>
-      </c>
-      <c r="J302">
-        <v>1</v>
       </c>
     </row>
     <row r="303" spans="1:10" x14ac:dyDescent="0.25">
@@ -10816,22 +10836,22 @@
         <v>2015</v>
       </c>
       <c r="C303" s="2">
-        <v>42317</v>
+        <v>42042</v>
       </c>
       <c r="D303" s="4">
         <f t="shared" si="28"/>
-        <v>2014</v>
+        <v>2013</v>
       </c>
       <c r="E303" s="4">
         <f t="shared" si="29"/>
-        <v>2013</v>
+        <v>2012</v>
       </c>
       <c r="F303">
-        <v>4151619</v>
+        <v>1210757</v>
       </c>
       <c r="G303">
-        <f>0.3*F303</f>
-        <v>1245485.7</v>
+        <f>F303*0.23</f>
+        <v>278474.11</v>
       </c>
       <c r="H303">
         <v>0</v>
@@ -10849,10 +10869,10 @@
       </c>
       <c r="B304">
         <f t="shared" si="25"/>
-        <v>2016</v>
+        <v>2015</v>
       </c>
       <c r="C304" s="2">
-        <v>42417</v>
+        <v>42317</v>
       </c>
       <c r="D304" s="4">
         <f t="shared" si="28"/>
@@ -10863,13 +10883,20 @@
         <v>2013</v>
       </c>
       <c r="F304">
-        <v>4150000</v>
+        <v>4151619</v>
+      </c>
+      <c r="G304">
+        <f>0.3*F304</f>
+        <v>1245485.7</v>
       </c>
       <c r="H304">
         <v>0</v>
       </c>
       <c r="I304">
         <v>0</v>
+      </c>
+      <c r="J304">
+        <v>1</v>
       </c>
     </row>
     <row r="305" spans="1:10" x14ac:dyDescent="0.25">
@@ -10881,30 +10908,24 @@
         <v>2016</v>
       </c>
       <c r="C305" s="2">
-        <v>42668</v>
+        <v>42417</v>
       </c>
       <c r="D305" s="4">
         <f t="shared" si="28"/>
-        <v>2015</v>
+        <v>2014</v>
       </c>
       <c r="E305" s="4">
         <f t="shared" si="29"/>
-        <v>2014</v>
+        <v>2013</v>
       </c>
       <c r="F305">
-        <v>5917285</v>
-      </c>
-      <c r="G305">
-        <v>1047465</v>
+        <v>4150000</v>
       </c>
       <c r="H305">
         <v>0</v>
       </c>
       <c r="I305">
         <v>0</v>
-      </c>
-      <c r="J305">
-        <v>1</v>
       </c>
     </row>
     <row r="306" spans="1:10" x14ac:dyDescent="0.25">
@@ -10913,31 +10934,33 @@
       </c>
       <c r="B306">
         <f t="shared" si="25"/>
-        <v>2017</v>
+        <v>2016</v>
       </c>
       <c r="C306" s="2">
-        <v>43056</v>
+        <v>42668</v>
       </c>
       <c r="D306" s="4">
         <f t="shared" si="28"/>
-        <v>2016</v>
+        <v>2015</v>
       </c>
       <c r="E306" s="4">
         <f t="shared" si="29"/>
-        <v>2015</v>
+        <v>2014</v>
       </c>
       <c r="F306">
-        <v>6423238</v>
+        <v>5917285</v>
       </c>
       <c r="G306">
-        <f>(6823499-6022976)/1.28</f>
-        <v>625408.59375</v>
+        <v>1047465</v>
       </c>
       <c r="H306">
         <v>0</v>
       </c>
       <c r="I306">
         <v>0</v>
+      </c>
+      <c r="J306">
+        <v>1</v>
       </c>
     </row>
     <row r="307" spans="1:10" x14ac:dyDescent="0.25">
@@ -10946,10 +10969,10 @@
       </c>
       <c r="B307">
         <f t="shared" si="25"/>
-        <v>2018</v>
+        <v>2017</v>
       </c>
       <c r="C307" s="2">
-        <v>43151</v>
+        <v>43056</v>
       </c>
       <c r="D307" s="4">
         <f t="shared" si="28"/>
@@ -10960,20 +10983,17 @@
         <v>2015</v>
       </c>
       <c r="F307">
-        <v>8422379</v>
+        <v>6423238</v>
       </c>
       <c r="G307">
-        <f>(8746816-8097942)/1.28</f>
-        <v>506932.8125</v>
+        <f>(6823499-6022976)/1.28</f>
+        <v>625408.59375</v>
       </c>
       <c r="H307">
         <v>0</v>
       </c>
       <c r="I307">
         <v>0</v>
-      </c>
-      <c r="J307">
-        <v>1</v>
       </c>
     </row>
     <row r="308" spans="1:10" x14ac:dyDescent="0.25">
@@ -10982,25 +11002,25 @@
       </c>
       <c r="B308">
         <f t="shared" si="25"/>
-        <v>2019</v>
+        <v>2018</v>
       </c>
       <c r="C308" s="2">
-        <v>43488</v>
+        <v>43151</v>
       </c>
       <c r="D308" s="4">
         <f t="shared" si="28"/>
-        <v>2017</v>
+        <v>2016</v>
       </c>
       <c r="E308" s="4">
         <f t="shared" si="29"/>
-        <v>2016</v>
+        <v>2015</v>
       </c>
       <c r="F308">
-        <v>1555655</v>
+        <v>8422379</v>
       </c>
       <c r="G308">
-        <f>(1633398-1477932)/1.28</f>
-        <v>121457.8125</v>
+        <f>(8746816-8097942)/1.28</f>
+        <v>506932.8125</v>
       </c>
       <c r="H308">
         <v>0</v>
@@ -11018,25 +11038,25 @@
       </c>
       <c r="B309">
         <f t="shared" si="25"/>
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="C309" s="2">
-        <v>43886</v>
+        <v>43488</v>
       </c>
       <c r="D309" s="4">
         <f t="shared" si="28"/>
-        <v>2018</v>
+        <v>2017</v>
       </c>
       <c r="E309" s="4">
         <f t="shared" si="29"/>
-        <v>2017</v>
+        <v>2016</v>
       </c>
       <c r="F309">
-        <v>3784000</v>
+        <v>1555655</v>
       </c>
       <c r="G309">
-        <f>(4243000-3362000)/1.96</f>
-        <v>449489.79591836734</v>
+        <f>(1633398-1477932)/1.28</f>
+        <v>121457.8125</v>
       </c>
       <c r="H309">
         <v>0</v>
@@ -11054,25 +11074,25 @@
       </c>
       <c r="B310">
         <f t="shared" si="25"/>
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C310" s="2">
-        <v>44243</v>
+        <v>43886</v>
       </c>
       <c r="D310" s="4">
         <f t="shared" si="28"/>
-        <v>2019</v>
+        <v>2018</v>
       </c>
       <c r="E310" s="4">
         <f t="shared" si="29"/>
-        <v>2018</v>
+        <v>2017</v>
       </c>
       <c r="F310">
-        <v>1630000</v>
+        <v>3784000</v>
       </c>
       <c r="G310">
-        <f>0.1*F310</f>
-        <v>163000</v>
+        <f>(4243000-3362000)/1.96</f>
+        <v>449489.79591836734</v>
       </c>
       <c r="H310">
         <v>0</v>
@@ -11090,32 +11110,31 @@
       </c>
       <c r="B311">
         <f t="shared" si="25"/>
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C311" s="2">
-        <v>44593</v>
+        <v>44243</v>
       </c>
       <c r="D311" s="4">
         <f t="shared" si="28"/>
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="E311" s="4">
         <f t="shared" si="29"/>
-        <v>2019</v>
+        <v>2018</v>
       </c>
       <c r="F311">
-        <v>2207921</v>
+        <v>1630000</v>
       </c>
       <c r="G311">
-        <f>(2432712-1999434)/1.96</f>
-        <v>221060.20408163266</v>
+        <f>0.1*F311</f>
+        <v>163000</v>
       </c>
       <c r="H311">
-        <v>16791</v>
+        <v>0</v>
       </c>
       <c r="I311">
-        <f>(18495-15205)/1.96</f>
-        <v>1678.5714285714287</v>
+        <v>0</v>
       </c>
       <c r="J311">
         <v>1</v>
@@ -11127,31 +11146,32 @@
       </c>
       <c r="B312">
         <f t="shared" si="25"/>
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C312" s="2">
-        <v>44970</v>
+        <v>44593</v>
       </c>
       <c r="D312" s="4">
         <f t="shared" si="28"/>
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="E312" s="4">
         <f t="shared" si="29"/>
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="F312">
-        <v>1219678</v>
+        <v>2207921</v>
       </c>
       <c r="G312">
-        <f>(1343499-1104508)/1.96</f>
-        <v>121934.18367346939</v>
+        <f>(2432712-1999434)/1.96</f>
+        <v>221060.20408163266</v>
       </c>
       <c r="H312">
-        <v>0</v>
+        <v>16791</v>
       </c>
       <c r="I312">
-        <v>0</v>
+        <f>(18495-15205)/1.96</f>
+        <v>1678.5714285714287</v>
       </c>
       <c r="J312">
         <v>1</v>
@@ -11162,27 +11182,63 @@
         <v>12</v>
       </c>
       <c r="B313">
+        <f t="shared" si="25"/>
+        <v>2023</v>
+      </c>
+      <c r="C313" s="2">
+        <v>44970</v>
+      </c>
+      <c r="D313" s="4">
+        <f t="shared" si="28"/>
+        <v>2021</v>
+      </c>
+      <c r="E313" s="4">
+        <f t="shared" si="29"/>
+        <v>2020</v>
+      </c>
+      <c r="F313">
+        <v>1219678</v>
+      </c>
+      <c r="G313">
+        <f>(1343499-1104508)/1.96</f>
+        <v>121934.18367346939</v>
+      </c>
+      <c r="H313">
+        <v>0</v>
+      </c>
+      <c r="I313">
+        <v>0</v>
+      </c>
+      <c r="J313">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="314" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A314" t="s">
+        <v>12</v>
+      </c>
+      <c r="B314">
         <v>2024</v>
       </c>
-      <c r="C313" s="2">
+      <c r="C314" s="2">
         <v>45357</v>
       </c>
-      <c r="D313" s="4">
-        <f>IF(MONTH(C313)&lt;4,B313-2,B313-1)</f>
+      <c r="D314" s="4">
+        <f>IF(MONTH(C314)&lt;4,B314-2,B314-1)</f>
         <v>2022</v>
       </c>
-      <c r="E313" s="4">
-        <f>IF(MONTH(C313)&lt;4,B313-3,B313-2)</f>
+      <c r="E314" s="4">
+        <f>IF(MONTH(C314)&lt;4,B314-3,B314-2)</f>
         <v>2021</v>
       </c>
-      <c r="F313">
+      <c r="F314">
         <v>1481384</v>
       </c>
-      <c r="G313">
+      <c r="G314">
         <f>(1642999-1331841)/1.96</f>
         <v>158754.08163265308</v>
       </c>
-      <c r="J313">
+      <c r="J314">
         <v>1</v>
       </c>
     </row>

</xml_diff>